<commit_message>
Hamburger UI change, Test cases change.
</commit_message>
<xml_diff>
--- a/src/global/utils/file-utils/locators(2).xlsx
+++ b/src/global/utils/file-utils/locators(2).xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="10"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="HomePage"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2898" uniqueCount="834">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2913" uniqueCount="841">
   <si>
     <t>page</t>
   </si>
@@ -1990,7 +1990,7 @@
     <t>myAccount</t>
   </si>
   <si>
-    <t>My Account</t>
+    <t>#My\ Profile-hamburger-menu-btn</t>
   </si>
   <si>
     <t>bettingRulesGHS</t>
@@ -2008,12 +2008,36 @@
     <t>bettingRulesMZ</t>
   </si>
   <si>
+    <t xml:space="preserve"> Betting Rules</t>
+  </si>
+  <si>
     <t>bettingRulesTips</t>
   </si>
   <si>
     <t>Betting Rules and Tips</t>
   </si>
   <si>
+    <t>insiderBlog</t>
+  </si>
+  <si>
+    <t>Insider Blog</t>
+  </si>
+  <si>
+    <t>betwayScoresApp</t>
+  </si>
+  <si>
+    <t>Betway Scores App</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>howTo</t>
+  </si>
+  <si>
+    <t>How To</t>
+  </si>
+  <si>
     <t>statistics</t>
   </si>
   <si>
@@ -2050,13 +2074,13 @@
     <t>depositFund</t>
   </si>
   <si>
-    <t>#Deposit\ funds-hamburger-menu-btn</t>
+    <t>{"name":"Deposit"}</t>
   </si>
   <si>
     <t>withdrawFund</t>
   </si>
   <si>
-    <t>#Withdraw\ funds-hamburger-menu-btn</t>
+    <t>{"name":"Withdraw"}</t>
   </si>
   <si>
     <t>closeWithdrawalAlert</t>
@@ -2107,7 +2131,7 @@
     <t>responsibleGaming</t>
   </si>
   <si>
-    <t>#Responsible\ Gaming-hamburger-menu-btn</t>
+    <t xml:space="preserve"> Responsible Gaming</t>
   </si>
   <si>
     <t>documentVerification</t>
@@ -2131,7 +2155,7 @@
     <t>changePassword</t>
   </si>
   <si>
-    <t>#Change\ password-hamburger-menu-btn</t>
+    <t>Change password details</t>
   </si>
   <si>
     <t>closeMyAccountOptions</t>
@@ -2218,9 +2242,6 @@
     <t>depositButton</t>
   </si>
   <si>
-    <t>{"name":"Deposit"}</t>
-  </si>
-  <si>
     <t>notificationBellIcon</t>
   </si>
   <si>
@@ -2248,7 +2269,7 @@
     <t>hide_closeDiveHam</t>
   </si>
   <si>
-    <t>//*[@id="__nuxt"]/div/div[1]/div[2]/div[1]/div[1]/div[1]/div[2]</t>
+    <t>/html/body/div[98]/div/div[2]/div/div/div[1]/div[1]/div[1]/div/details/summary/div/div[1]/div[2]</t>
   </si>
   <si>
     <t>liveChatIcon</t>
@@ -2541,7 +2562,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2611,6 +2632,12 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -2708,7 +2735,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="50">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2785,17 +2812,11 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="12" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2803,37 +2824,55 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="12" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="13" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="13" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="12" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="13" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="17" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="17" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="18" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="18" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="17" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="18" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="17" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
@@ -2842,7 +2881,7 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="18" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="19" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -3174,16 +3213,16 @@
       <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="43" t="s">
+      <c r="F1" s="47" t="s">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>798</v>
+        <v>805</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>8</v>
@@ -3192,7 +3231,7 @@
         <v>30</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>799</v>
+        <v>806</v>
       </c>
       <c r="F2" s="8">
         <v>1</v>
@@ -3200,10 +3239,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>800</v>
+        <v>807</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>8</v>
@@ -3212,22 +3251,22 @@
         <v>30</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>801</v>
+        <v>808</v>
       </c>
       <c r="F3" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>802</v>
+        <v>809</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>803</v>
+        <v>810</v>
       </c>
       <c r="E4" s="25" t="s">
         <v>23</v>
@@ -3236,10 +3275,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>804</v>
+        <v>811</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>8</v>
@@ -3248,16 +3287,16 @@
         <v>30</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>805</v>
+        <v>812</v>
       </c>
       <c r="F5" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>806</v>
+        <v>813</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>8</v>
@@ -3266,16 +3305,16 @@
         <v>30</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>807</v>
+        <v>814</v>
       </c>
       <c r="F6" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>808</v>
+        <v>815</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>8</v>
@@ -3284,22 +3323,22 @@
         <v>30</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>809</v>
+        <v>816</v>
       </c>
       <c r="F7" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>810</v>
+        <v>817</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>811</v>
+        <v>818</v>
       </c>
       <c r="E8" s="25" t="s">
         <v>23</v>
@@ -3308,16 +3347,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>812</v>
+        <v>819</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>813</v>
+        <v>820</v>
       </c>
       <c r="E9" s="25" t="s">
         <v>23</v>
@@ -3326,16 +3365,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>814</v>
+        <v>821</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>815</v>
+        <v>822</v>
       </c>
       <c r="E10" s="25" t="s">
         <v>23</v>
@@ -3344,10 +3383,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>816</v>
+        <v>823</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>8</v>
@@ -3356,22 +3395,22 @@
         <v>30</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>817</v>
+        <v>824</v>
       </c>
       <c r="F11" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>818</v>
+        <v>825</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>819</v>
+        <v>826</v>
       </c>
       <c r="E12" s="25" t="s">
         <v>23</v>
@@ -3380,16 +3419,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>820</v>
+        <v>827</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>820</v>
+        <v>827</v>
       </c>
       <c r="E13" s="25" t="s">
         <v>23</v>
@@ -3398,16 +3437,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>821</v>
+        <v>828</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>822</v>
+        <v>829</v>
       </c>
       <c r="E14" s="25" t="s">
         <v>23</v>
@@ -3416,16 +3455,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>823</v>
+        <v>830</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>824</v>
+        <v>831</v>
       </c>
       <c r="E15" s="25" t="s">
         <v>23</v>
@@ -3434,16 +3473,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>825</v>
+        <v>832</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>826</v>
+        <v>833</v>
       </c>
       <c r="E16" s="25" t="s">
         <v>23</v>
@@ -3452,16 +3491,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>827</v>
+        <v>834</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>828</v>
+        <v>835</v>
       </c>
       <c r="E17" s="25" t="s">
         <v>23</v>
@@ -3470,16 +3509,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>829</v>
+        <v>836</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>830</v>
+        <v>837</v>
       </c>
       <c r="E18" s="25" t="s">
         <v>23</v>
@@ -3488,16 +3527,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>831</v>
+        <v>838</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="45" t="s">
-        <v>832</v>
+      <c r="D19" s="49" t="s">
+        <v>839</v>
       </c>
       <c r="E19" s="25" t="s">
         <v>23</v>
@@ -3506,10 +3545,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="6" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>833</v>
+        <v>840</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>8</v>
@@ -3518,7 +3557,7 @@
         <v>30</v>
       </c>
       <c r="E20" s="25" t="s">
-        <v>799</v>
+        <v>806</v>
       </c>
       <c r="F20" s="8"/>
     </row>
@@ -10919,13 +10958,13 @@
       <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="43" t="s">
+      <c r="F1" s="47" t="s">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>176</v>
@@ -10945,7 +10984,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>187</v>
@@ -10957,7 +10996,7 @@
         <v>30</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>787</v>
+        <v>794</v>
       </c>
       <c r="F3" s="8">
         <v>0</v>
@@ -10965,7 +11004,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>189</v>
@@ -10985,7 +11024,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>191</v>
@@ -11005,7 +11044,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>193</v>
@@ -11025,7 +11064,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>195</v>
@@ -11045,7 +11084,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>197</v>
@@ -11057,7 +11096,7 @@
         <v>30</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>788</v>
+        <v>795</v>
       </c>
       <c r="F8" s="8">
         <v>0</v>
@@ -11065,7 +11104,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>199</v>
@@ -11077,7 +11116,7 @@
         <v>30</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>789</v>
+        <v>796</v>
       </c>
       <c r="F9" s="8">
         <v>0</v>
@@ -11085,7 +11124,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>201</v>
@@ -11097,7 +11136,7 @@
         <v>30</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>790</v>
+        <v>797</v>
       </c>
       <c r="F10" s="8">
         <v>0</v>
@@ -11105,7 +11144,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>203</v>
@@ -11117,7 +11156,7 @@
         <v>30</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>791</v>
+        <v>798</v>
       </c>
       <c r="F11" s="8">
         <v>0</v>
@@ -11125,7 +11164,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>205</v>
@@ -11137,7 +11176,7 @@
         <v>30</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>792</v>
+        <v>799</v>
       </c>
       <c r="F12" s="8">
         <v>0</v>
@@ -11145,7 +11184,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>207</v>
@@ -11157,7 +11196,7 @@
         <v>30</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>793</v>
+        <v>800</v>
       </c>
       <c r="F13" s="8">
         <v>0</v>
@@ -11165,7 +11204,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>209</v>
@@ -11185,7 +11224,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>211</v>
@@ -11197,7 +11236,7 @@
         <v>30</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="F15" s="8">
         <v>0</v>
@@ -11205,7 +11244,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>213</v>
@@ -11217,7 +11256,7 @@
         <v>30</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>795</v>
+        <v>802</v>
       </c>
       <c r="F16" s="8">
         <v>0</v>
@@ -11225,7 +11264,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>215</v>
@@ -11237,7 +11276,7 @@
         <v>30</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>796</v>
+        <v>803</v>
       </c>
       <c r="F17" s="8">
         <v>0</v>
@@ -11245,7 +11284,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>217</v>
@@ -11265,7 +11304,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>384</v>
@@ -11285,7 +11324,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>220</v>
@@ -11305,7 +11344,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>221</v>
@@ -11325,7 +11364,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>32</v>
@@ -11345,7 +11384,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>223</v>
@@ -11365,7 +11404,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>225</v>
@@ -11385,7 +11424,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>227</v>
@@ -11405,7 +11444,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="6" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>229</v>
@@ -11502,7 +11541,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>785</v>
+        <v>792</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>23</v>
@@ -11550,13 +11589,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="14" t="s">
-        <v>766</v>
+        <v>773</v>
       </c>
       <c r="B2" s="14" t="s">
         <v>68</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>767</v>
+        <v>774</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>23</v>
@@ -11567,13 +11606,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="14" t="s">
-        <v>768</v>
+        <v>775</v>
       </c>
       <c r="B3" s="14" t="s">
         <v>68</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>769</v>
+        <v>776</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>23</v>
@@ -11582,13 +11621,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="14" t="s">
-        <v>770</v>
+        <v>777</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>68</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>771</v>
+        <v>778</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>23</v>
@@ -11597,13 +11636,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="14" t="s">
-        <v>772</v>
+        <v>779</v>
       </c>
       <c r="B5" s="14" t="s">
         <v>68</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>773</v>
+        <v>780</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>23</v>
@@ -11612,13 +11651,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="14" t="s">
-        <v>774</v>
+        <v>781</v>
       </c>
       <c r="B6" s="14" t="s">
         <v>68</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>775</v>
+        <v>782</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>23</v>
@@ -11633,7 +11672,7 @@
         <v>21</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>776</v>
+        <v>783</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>23</v>
@@ -11642,13 +11681,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="6" t="s">
-        <v>777</v>
+        <v>784</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>778</v>
+        <v>785</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>23</v>
@@ -11657,13 +11696,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="6" t="s">
-        <v>779</v>
+        <v>786</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="44" t="s">
-        <v>780</v>
+      <c r="C9" s="48" t="s">
+        <v>787</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>23</v>
@@ -11672,13 +11711,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="6" t="s">
-        <v>781</v>
+        <v>788</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>68</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>782</v>
+        <v>789</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>23</v>
@@ -11687,7 +11726,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="6" t="s">
-        <v>783</v>
+        <v>790</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>8</v>
@@ -11696,7 +11735,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>784</v>
+        <v>791</v>
       </c>
       <c r="E11" s="8"/>
     </row>
@@ -11733,7 +11772,7 @@
       <c r="D1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="43" t="s">
+      <c r="E1" s="47" t="s">
         <v>5</v>
       </c>
     </row>
@@ -11765,7 +11804,7 @@
         <v>9</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>765</v>
+        <v>772</v>
       </c>
       <c r="E3" s="15">
         <v>0</v>
@@ -12416,274 +12455,274 @@
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="36" t="s">
+      <c r="A1" s="39" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="36" t="s">
+      <c r="C1" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="36" t="s">
+      <c r="D1" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="36" t="s">
+      <c r="E1" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="37" t="s">
+      <c r="F1" s="41" t="s">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B2" s="39" t="s">
-        <v>742</v>
-      </c>
-      <c r="C2" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="39" t="s">
+      <c r="A2" s="42" t="s">
+        <v>748</v>
+      </c>
+      <c r="B2" s="43" t="s">
+        <v>749</v>
+      </c>
+      <c r="C2" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="39" t="s">
-        <v>743</v>
-      </c>
-      <c r="F2" s="40">
+      <c r="E2" s="43" t="s">
+        <v>750</v>
+      </c>
+      <c r="F2" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B3" s="39" t="s">
-        <v>744</v>
-      </c>
-      <c r="C3" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="39" t="s">
+      <c r="A3" s="42" t="s">
+        <v>748</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>751</v>
+      </c>
+      <c r="C3" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="39" t="s">
-        <v>745</v>
-      </c>
-      <c r="F3" s="40">
+      <c r="E3" s="43" t="s">
+        <v>752</v>
+      </c>
+      <c r="F3" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B4" s="39" t="s">
-        <v>746</v>
-      </c>
-      <c r="C4" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="39" t="s">
-        <v>747</v>
-      </c>
-      <c r="E4" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="41"/>
+      <c r="A4" s="42" t="s">
+        <v>748</v>
+      </c>
+      <c r="B4" s="43" t="s">
+        <v>753</v>
+      </c>
+      <c r="C4" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="43" t="s">
+        <v>754</v>
+      </c>
+      <c r="E4" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="45"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B5" s="39" t="s">
+      <c r="A5" s="42" t="s">
         <v>748</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="B5" s="43" t="s">
+        <v>755</v>
+      </c>
+      <c r="C5" s="43" t="s">
         <v>68</v>
       </c>
-      <c r="D5" s="39" t="s">
-        <v>749</v>
-      </c>
-      <c r="E5" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="40">
+      <c r="D5" s="43" t="s">
+        <v>756</v>
+      </c>
+      <c r="E5" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B6" s="39" t="s">
-        <v>750</v>
-      </c>
-      <c r="C6" s="39" t="s">
+      <c r="A6" s="42" t="s">
+        <v>748</v>
+      </c>
+      <c r="B6" s="43" t="s">
+        <v>757</v>
+      </c>
+      <c r="C6" s="43" t="s">
         <v>68</v>
       </c>
-      <c r="D6" s="39" t="s">
-        <v>751</v>
-      </c>
-      <c r="E6" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="40">
+      <c r="D6" s="43" t="s">
+        <v>758</v>
+      </c>
+      <c r="E6" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B7" s="39" t="s">
-        <v>752</v>
-      </c>
-      <c r="C7" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="39" t="s">
-        <v>753</v>
-      </c>
-      <c r="E7" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="41"/>
+      <c r="A7" s="42" t="s">
+        <v>748</v>
+      </c>
+      <c r="B7" s="43" t="s">
+        <v>759</v>
+      </c>
+      <c r="C7" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="43" t="s">
+        <v>760</v>
+      </c>
+      <c r="E7" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="45"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B8" s="39" t="s">
-        <v>754</v>
-      </c>
-      <c r="C8" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="39" t="s">
-        <v>755</v>
-      </c>
-      <c r="E8" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="41"/>
+      <c r="A8" s="42" t="s">
+        <v>748</v>
+      </c>
+      <c r="B8" s="43" t="s">
+        <v>761</v>
+      </c>
+      <c r="C8" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>762</v>
+      </c>
+      <c r="E8" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="45"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B9" s="39" t="s">
-        <v>756</v>
-      </c>
-      <c r="C9" s="39" t="s">
+      <c r="A9" s="42" t="s">
+        <v>748</v>
+      </c>
+      <c r="B9" s="43" t="s">
+        <v>763</v>
+      </c>
+      <c r="C9" s="43" t="s">
         <v>68</v>
       </c>
-      <c r="D9" s="39" t="s">
-        <v>757</v>
-      </c>
-      <c r="E9" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" s="40">
+      <c r="D9" s="43" t="s">
+        <v>764</v>
+      </c>
+      <c r="E9" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B10" s="39" t="s">
-        <v>758</v>
-      </c>
-      <c r="C10" s="39" t="s">
+      <c r="A10" s="42" t="s">
+        <v>748</v>
+      </c>
+      <c r="B10" s="43" t="s">
+        <v>765</v>
+      </c>
+      <c r="C10" s="43" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="39" t="s">
-        <v>759</v>
-      </c>
-      <c r="E10" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="40">
+      <c r="D10" s="43" t="s">
+        <v>766</v>
+      </c>
+      <c r="E10" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B11" s="39" t="s">
+      <c r="A11" s="42" t="s">
+        <v>748</v>
+      </c>
+      <c r="B11" s="43" t="s">
         <v>489</v>
       </c>
-      <c r="C11" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="39" t="s">
-        <v>760</v>
-      </c>
-      <c r="E11" s="39" t="s">
+      <c r="C11" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="43" t="s">
+        <v>767</v>
+      </c>
+      <c r="E11" s="43" t="s">
         <v>490</v>
       </c>
-      <c r="F11" s="40">
+      <c r="F11" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B12" s="39" t="s">
+      <c r="A12" s="42" t="s">
+        <v>748</v>
+      </c>
+      <c r="B12" s="43" t="s">
         <v>491</v>
       </c>
-      <c r="C12" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="39" t="s">
-        <v>760</v>
-      </c>
-      <c r="E12" s="39" t="s">
+      <c r="C12" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="43" t="s">
+        <v>767</v>
+      </c>
+      <c r="E12" s="43" t="s">
         <v>492</v>
       </c>
-      <c r="F12" s="40">
+      <c r="F12" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B13" s="39" t="s">
-        <v>761</v>
-      </c>
-      <c r="C13" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="39" t="s">
-        <v>762</v>
-      </c>
-      <c r="E13" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" s="41"/>
+      <c r="A13" s="42" t="s">
+        <v>748</v>
+      </c>
+      <c r="B13" s="43" t="s">
+        <v>768</v>
+      </c>
+      <c r="C13" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="43" t="s">
+        <v>769</v>
+      </c>
+      <c r="E13" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" s="45"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="38" t="s">
-        <v>741</v>
-      </c>
-      <c r="B14" s="38" t="s">
-        <v>763</v>
-      </c>
-      <c r="C14" s="38" t="s">
+      <c r="A14" s="42" t="s">
+        <v>748</v>
+      </c>
+      <c r="B14" s="42" t="s">
+        <v>770</v>
+      </c>
+      <c r="C14" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="D14" s="38" t="s">
-        <v>764</v>
-      </c>
-      <c r="E14" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="42">
+      <c r="D14" s="42" t="s">
+        <v>771</v>
+      </c>
+      <c r="E14" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="46">
         <v>0</v>
       </c>
     </row>
@@ -12697,7 +12736,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="4" width="12.290714285714287" customWidth="1" bestFit="1"/>
@@ -12952,7 +12991,9 @@
       <c r="E13" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F13" s="16"/>
+      <c r="F13" s="16">
+        <v>0</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="17" t="s">
@@ -12962,7 +13003,7 @@
         <v>651</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="D14" s="34" t="s">
         <v>652</v>
@@ -13039,25 +13080,27 @@
         <v>68</v>
       </c>
       <c r="D18" s="34" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="E18" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F18" s="16"/>
+      <c r="F18" s="16">
+        <v>0</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C19" s="17" t="s">
         <v>68</v>
       </c>
       <c r="D19" s="34" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="E19" s="17" t="s">
         <v>23</v>
@@ -13068,57 +13111,53 @@
       <c r="A20" s="17" t="s">
         <v>643</v>
       </c>
-      <c r="B20" s="17" t="s">
-        <v>660</v>
+      <c r="B20" s="35" t="s">
+        <v>661</v>
       </c>
       <c r="C20" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="D20" s="34" t="s">
-        <v>661</v>
-      </c>
-      <c r="E20" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="F20" s="18">
-        <v>0</v>
-      </c>
+      <c r="D20" s="36" t="s">
+        <v>662</v>
+      </c>
+      <c r="E20" s="35"/>
+      <c r="F20" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="17" t="s">
         <v>643</v>
       </c>
-      <c r="B21" s="17" t="s">
-        <v>662</v>
+      <c r="B21" s="35" t="s">
+        <v>663</v>
       </c>
       <c r="C21" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="D21" s="34" t="s">
-        <v>663</v>
-      </c>
-      <c r="E21" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="F21" s="16"/>
+      <c r="D21" s="36" t="s">
+        <v>664</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>665</v>
+      </c>
+      <c r="F21" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="D22" s="18">
-        <v>27</v>
+      <c r="D22" s="34" t="s">
+        <v>667</v>
       </c>
       <c r="E22" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F22" s="16">
+      <c r="F22" s="18">
         <v>0</v>
       </c>
     </row>
@@ -13127,31 +13166,33 @@
         <v>643</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="D23" s="34" t="s">
-        <v>381</v>
+        <v>669</v>
       </c>
       <c r="E23" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F23" s="16"/>
+      <c r="F23" s="18">
+        <v>0</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>165</v>
+        <v>670</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="D24" s="34" t="s">
-        <v>382</v>
+        <v>671</v>
       </c>
       <c r="E24" s="17" t="s">
         <v>23</v>
@@ -13163,31 +13204,33 @@
         <v>643</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="D25" s="34" t="s">
-        <v>667</v>
+        <v>68</v>
+      </c>
+      <c r="D25" s="18">
+        <v>27</v>
       </c>
       <c r="E25" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F25" s="16"/>
+      <c r="F25" s="16">
+        <v>0</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="D26" s="34" t="s">
-        <v>669</v>
+        <v>381</v>
       </c>
       <c r="E26" s="17" t="s">
         <v>23</v>
@@ -13199,13 +13242,13 @@
         <v>643</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>384</v>
+        <v>165</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="D27" s="34" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="E27" s="17" t="s">
         <v>23</v>
@@ -13217,16 +13260,16 @@
         <v>643</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="D28" s="34" t="s">
-        <v>14</v>
+        <v>675</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>75</v>
+        <v>23</v>
       </c>
       <c r="F28" s="16"/>
     </row>
@@ -13235,31 +13278,33 @@
         <v>643</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="D29" s="34" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="E29" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F29" s="16"/>
+      <c r="F29" s="38" t="s">
+        <v>665</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>673</v>
+        <v>384</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="D30" s="34" t="s">
-        <v>674</v>
+        <v>385</v>
       </c>
       <c r="E30" s="17" t="s">
         <v>23</v>
@@ -13271,54 +13316,54 @@
         <v>643</v>
       </c>
       <c r="B31" s="17" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D31" s="34" t="s">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="E31" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="F31" s="18">
-        <v>1</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="F31" s="16"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D32" s="34" t="s">
-        <v>677</v>
+        <v>14</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="F32" s="16"/>
+        <v>680</v>
+      </c>
+      <c r="F32" s="16">
+        <v>1</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B33" s="17" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D33" s="34" t="s">
-        <v>679</v>
+        <v>14</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>23</v>
+        <v>682</v>
       </c>
       <c r="F33" s="16"/>
     </row>
@@ -13327,31 +13372,33 @@
         <v>643</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="D34" s="34" t="s">
-        <v>681</v>
+        <v>77</v>
       </c>
       <c r="E34" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F34" s="16"/>
+      <c r="F34" s="18">
+        <v>1</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="D35" s="34" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="E35" s="17" t="s">
         <v>23</v>
@@ -13363,13 +13410,13 @@
         <v>643</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="D36" s="34" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="E36" s="17" t="s">
         <v>23</v>
@@ -13381,13 +13428,13 @@
         <v>643</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>184</v>
+        <v>688</v>
       </c>
       <c r="C37" s="17" t="s">
         <v>68</v>
       </c>
       <c r="D37" s="34" t="s">
-        <v>185</v>
+        <v>689</v>
       </c>
       <c r="E37" s="17" t="s">
         <v>23</v>
@@ -13399,13 +13446,13 @@
         <v>643</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="C38" s="17" t="s">
         <v>68</v>
       </c>
       <c r="D38" s="34" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="E38" s="17" t="s">
         <v>23</v>
@@ -13417,13 +13464,13 @@
         <v>643</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="C39" s="17" t="s">
         <v>68</v>
       </c>
       <c r="D39" s="34" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="E39" s="17" t="s">
         <v>23</v>
@@ -13435,13 +13482,13 @@
         <v>643</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>690</v>
+        <v>184</v>
       </c>
       <c r="C40" s="17" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="D40" s="34" t="s">
-        <v>691</v>
+        <v>185</v>
       </c>
       <c r="E40" s="17" t="s">
         <v>23</v>
@@ -13453,13 +13500,13 @@
         <v>643</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="C41" s="17" t="s">
         <v>68</v>
       </c>
       <c r="D41" s="34" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="E41" s="17" t="s">
         <v>23</v>
@@ -13471,13 +13518,13 @@
         <v>643</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="C42" s="17" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="D42" s="34" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="E42" s="17" t="s">
         <v>23</v>
@@ -13489,31 +13536,33 @@
         <v>643</v>
       </c>
       <c r="B43" s="17" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="C43" s="17" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="D43" s="34" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="E43" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F43" s="16"/>
+      <c r="F43" s="16">
+        <v>0</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
       <c r="A44" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="D44" s="34" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="E44" s="17" t="s">
         <v>23</v>
@@ -13525,13 +13574,13 @@
         <v>643</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>639</v>
+        <v>702</v>
       </c>
       <c r="C45" s="17" t="s">
         <v>21</v>
       </c>
       <c r="D45" s="34" t="s">
-        <v>640</v>
+        <v>703</v>
       </c>
       <c r="E45" s="17" t="s">
         <v>23</v>
@@ -13543,33 +13592,31 @@
         <v>643</v>
       </c>
       <c r="B46" s="17" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="C46" s="17" t="s">
         <v>21</v>
       </c>
       <c r="D46" s="34" t="s">
-        <v>77</v>
+        <v>705</v>
       </c>
       <c r="E46" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F46" s="18">
-        <v>1</v>
-      </c>
+      <c r="F46" s="16"/>
     </row>
     <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
       <c r="A47" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B47" s="17" t="s">
-        <v>701</v>
+        <v>706</v>
       </c>
       <c r="C47" s="17" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="D47" s="34" t="s">
-        <v>702</v>
+        <v>707</v>
       </c>
       <c r="E47" s="17" t="s">
         <v>23</v>
@@ -13581,39 +13628,37 @@
         <v>643</v>
       </c>
       <c r="B48" s="17" t="s">
-        <v>703</v>
+        <v>639</v>
       </c>
       <c r="C48" s="17" t="s">
         <v>21</v>
       </c>
       <c r="D48" s="34" t="s">
-        <v>704</v>
+        <v>640</v>
       </c>
       <c r="E48" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F48" s="18">
-        <v>0</v>
-      </c>
+      <c r="F48" s="16"/>
     </row>
     <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
       <c r="A49" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B49" s="17" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
       <c r="C49" s="17" t="s">
         <v>21</v>
       </c>
       <c r="D49" s="34" t="s">
-        <v>706</v>
+        <v>77</v>
       </c>
       <c r="E49" s="17" t="s">
         <v>23</v>
       </c>
       <c r="F49" s="18">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
@@ -13621,16 +13666,16 @@
         <v>643</v>
       </c>
       <c r="B50" s="17" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="C50" s="17" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="D50" s="34" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="E50" s="17" t="s">
-        <v>162</v>
+        <v>23</v>
       </c>
       <c r="F50" s="16"/>
     </row>
@@ -13639,52 +13684,56 @@
         <v>643</v>
       </c>
       <c r="B51" s="17" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="C51" s="17" t="s">
         <v>21</v>
       </c>
       <c r="D51" s="34" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="E51" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F51" s="34"/>
+      <c r="F51" s="18">
+        <v>0</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
       <c r="A52" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="C52" s="17" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D52" s="34" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="E52" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F52" s="16"/>
+      <c r="F52" s="18">
+        <v>0</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
       <c r="A53" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B53" s="17" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="C53" s="17" t="s">
         <v>68</v>
       </c>
       <c r="D53" s="34" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="E53" s="17" t="s">
-        <v>23</v>
+        <v>162</v>
       </c>
       <c r="F53" s="16"/>
     </row>
@@ -13693,31 +13742,31 @@
         <v>643</v>
       </c>
       <c r="B54" s="17" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="C54" s="17" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="D54" s="34" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="E54" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F54" s="16"/>
+      <c r="F54" s="34"/>
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
       <c r="A55" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="C55" s="17" t="s">
-        <v>68</v>
+        <v>25</v>
       </c>
       <c r="D55" s="34" t="s">
-        <v>714</v>
+        <v>720</v>
       </c>
       <c r="E55" s="17" t="s">
         <v>23</v>
@@ -13729,13 +13778,13 @@
         <v>643</v>
       </c>
       <c r="B56" s="17" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="C56" s="17" t="s">
-        <v>719</v>
+        <v>68</v>
       </c>
       <c r="D56" s="34" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="E56" s="17" t="s">
         <v>23</v>
@@ -13747,13 +13796,13 @@
         <v>643</v>
       </c>
       <c r="B57" s="17" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="C57" s="17" t="s">
         <v>68</v>
       </c>
       <c r="D57" s="34" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="E57" s="17" t="s">
         <v>23</v>
@@ -13765,7 +13814,7 @@
         <v>643</v>
       </c>
       <c r="B58" s="17" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="C58" s="17" t="s">
         <v>68</v>
@@ -13776,22 +13825,20 @@
       <c r="E58" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F58" s="18">
-        <v>1</v>
-      </c>
+      <c r="F58" s="16"/>
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
       <c r="A59" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B59" s="17" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="C59" s="17" t="s">
-        <v>68</v>
+        <v>727</v>
       </c>
       <c r="D59" s="34" t="s">
-        <v>714</v>
+        <v>728</v>
       </c>
       <c r="E59" s="17" t="s">
         <v>23</v>
@@ -13803,51 +13850,51 @@
         <v>643</v>
       </c>
       <c r="B60" s="17" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="C60" s="17" t="s">
-        <v>719</v>
+        <v>68</v>
       </c>
       <c r="D60" s="34" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="E60" s="17" t="s">
         <v>23</v>
       </c>
       <c r="F60" s="16"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
       <c r="A61" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B61" s="17" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="C61" s="17" t="s">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="D61" s="34" t="s">
-        <v>14</v>
+        <v>730</v>
       </c>
       <c r="E61" s="17" t="s">
-        <v>728</v>
+        <v>23</v>
       </c>
       <c r="F61" s="18">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
       <c r="A62" s="17" t="s">
         <v>643</v>
       </c>
       <c r="B62" s="17" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
       <c r="C62" s="17" t="s">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="D62" s="34" t="s">
-        <v>730</v>
+        <v>722</v>
       </c>
       <c r="E62" s="17" t="s">
         <v>23</v>
@@ -13859,90 +13906,146 @@
         <v>643</v>
       </c>
       <c r="B63" s="17" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="C63" s="17" t="s">
+        <v>727</v>
+      </c>
+      <c r="D63" s="34" t="s">
+        <v>734</v>
+      </c>
+      <c r="E63" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F63" s="16"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="19.5">
+      <c r="A64" s="17" t="s">
+        <v>643</v>
+      </c>
+      <c r="B64" s="17" t="s">
+        <v>735</v>
+      </c>
+      <c r="C64" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D64" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="E64" s="17" t="s">
+        <v>680</v>
+      </c>
+      <c r="F64" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="19.5">
+      <c r="A65" s="17" t="s">
+        <v>643</v>
+      </c>
+      <c r="B65" s="17" t="s">
+        <v>736</v>
+      </c>
+      <c r="C65" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D65" s="34" t="s">
+        <v>737</v>
+      </c>
+      <c r="E65" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F65" s="16"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
+      <c r="A66" s="17" t="s">
+        <v>643</v>
+      </c>
+      <c r="B66" s="17" t="s">
+        <v>738</v>
+      </c>
+      <c r="C66" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="D63" s="34" t="s">
-        <v>732</v>
-      </c>
-      <c r="E63" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="F63" s="16"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
-      <c r="A64" s="25" t="s">
+      <c r="D66" s="34" t="s">
+        <v>739</v>
+      </c>
+      <c r="E66" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F66" s="16"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
+      <c r="A67" s="25" t="s">
         <v>643</v>
       </c>
-      <c r="B64" s="25" t="s">
-        <v>733</v>
-      </c>
-      <c r="C64" s="25" t="s">
+      <c r="B67" s="25" t="s">
+        <v>740</v>
+      </c>
+      <c r="C67" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="D64" s="7" t="s">
-        <v>734</v>
-      </c>
-      <c r="E64" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="F64" s="7"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
-      <c r="A65" s="25" t="s">
+      <c r="D67" s="7" t="s">
+        <v>741</v>
+      </c>
+      <c r="E67" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="F67" s="7"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
+      <c r="A68" s="25" t="s">
         <v>643</v>
       </c>
-      <c r="B65" s="25" t="s">
-        <v>735</v>
-      </c>
-      <c r="C65" s="25" t="s">
+      <c r="B68" s="25" t="s">
+        <v>742</v>
+      </c>
+      <c r="C68" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="D65" s="7" t="s">
-        <v>736</v>
-      </c>
-      <c r="E65" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="F65" s="7"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
-      <c r="A66" s="25" t="s">
+      <c r="D68" s="7" t="s">
+        <v>743</v>
+      </c>
+      <c r="E68" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="F68" s="7"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
+      <c r="A69" s="25" t="s">
         <v>643</v>
       </c>
-      <c r="B66" s="25" t="s">
-        <v>737</v>
-      </c>
-      <c r="C66" s="25" t="s">
+      <c r="B69" s="25" t="s">
+        <v>744</v>
+      </c>
+      <c r="C69" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="D66" s="7" t="s">
-        <v>738</v>
-      </c>
-      <c r="E66" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="F66" s="7"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="19.5">
-      <c r="A67" s="17" t="s">
+      <c r="D69" s="7" t="s">
+        <v>745</v>
+      </c>
+      <c r="E69" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="F69" s="7"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="19.5">
+      <c r="A70" s="17" t="s">
         <v>643</v>
       </c>
-      <c r="B67" s="17" t="s">
-        <v>739</v>
-      </c>
-      <c r="C67" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="D67" s="34" t="s">
-        <v>740</v>
-      </c>
-      <c r="E67" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="F67" s="16"/>
+      <c r="B70" s="17" t="s">
+        <v>746</v>
+      </c>
+      <c r="C70" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="D70" s="34" t="s">
+        <v>747</v>
+      </c>
+      <c r="E70" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F70" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix some test cases after ui change in website
</commit_message>
<xml_diff>
--- a/src/global/utils/file-utils/locators(2).xlsx
+++ b/src/global/utils/file-utils/locators(2).xlsx
@@ -2026,19 +2026,19 @@
     <t>betwayScoresApp</t>
   </si>
   <si>
-    <t>Betway Scores App</t>
+    <t xml:space="preserve"> Betway Scores App</t>
   </si>
   <si>
     <t>howTo</t>
   </si>
   <si>
-    <t>How To</t>
+    <t>{"name":"How To","exact":true}</t>
   </si>
   <si>
     <t>statistics</t>
   </si>
   <si>
-    <t>Statistics</t>
+    <t>{"name":"Statistics"}</t>
   </si>
   <si>
     <t>oddsFormat</t>
@@ -2128,7 +2128,7 @@
     <t>responsibleGaming</t>
   </si>
   <si>
-    <t xml:space="preserve"> Responsible Gaming</t>
+    <t>#Responsible\ Gaming-hamburger-menu-btn</t>
   </si>
   <si>
     <t>documentVerification</t>
@@ -2161,7 +2161,7 @@
     <t>hamburgerEyeButton</t>
   </si>
   <si>
-    <t>(.w-6.h-6.cursor-pointer &gt; path').first()</t>
+    <t>div.mr-2 &gt; svg.w-6.h-6.cursor-pointer</t>
   </si>
   <si>
     <t>accountsButtonMZ</t>
@@ -2559,7 +2559,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2651,12 +2651,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2732,7 +2726,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="44">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2831,33 +2825,27 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="17" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="18" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="17" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="17" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="18" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="18" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="17" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
@@ -2866,7 +2854,7 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="19" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="18" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -3198,11 +3186,11 @@
       <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="43" t="s">
+      <c r="F1" s="41" t="s">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="6" t="s">
         <v>803</v>
       </c>
@@ -3222,7 +3210,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="6" t="s">
         <v>803</v>
       </c>
@@ -3240,7 +3228,7 @@
       </c>
       <c r="F3" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="6" t="s">
         <v>803</v>
       </c>
@@ -3258,7 +3246,7 @@
       </c>
       <c r="F4" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="6" t="s">
         <v>803</v>
       </c>
@@ -3276,7 +3264,7 @@
       </c>
       <c r="F5" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="6" t="s">
         <v>803</v>
       </c>
@@ -3294,7 +3282,7 @@
       </c>
       <c r="F6" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="6" t="s">
         <v>803</v>
       </c>
@@ -3312,7 +3300,7 @@
       </c>
       <c r="F7" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="6" t="s">
         <v>803</v>
       </c>
@@ -3330,7 +3318,7 @@
       </c>
       <c r="F8" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="6" t="s">
         <v>803</v>
       </c>
@@ -3348,7 +3336,7 @@
       </c>
       <c r="F9" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="6" t="s">
         <v>803</v>
       </c>
@@ -3366,7 +3354,7 @@
       </c>
       <c r="F10" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="6" t="s">
         <v>803</v>
       </c>
@@ -3382,9 +3370,11 @@
       <c r="E11" s="25" t="s">
         <v>823</v>
       </c>
-      <c r="F11" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="F11" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="6" t="s">
         <v>803</v>
       </c>
@@ -3402,7 +3392,7 @@
       </c>
       <c r="F12" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="6" t="s">
         <v>803</v>
       </c>
@@ -3420,7 +3410,7 @@
       </c>
       <c r="F13" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="6" t="s">
         <v>803</v>
       </c>
@@ -3438,7 +3428,7 @@
       </c>
       <c r="F14" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="6" t="s">
         <v>803</v>
       </c>
@@ -3456,7 +3446,7 @@
       </c>
       <c r="F15" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="6" t="s">
         <v>803</v>
       </c>
@@ -3474,7 +3464,7 @@
       </c>
       <c r="F16" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="6" t="s">
         <v>803</v>
       </c>
@@ -3492,7 +3482,7 @@
       </c>
       <c r="F17" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="6" t="s">
         <v>803</v>
       </c>
@@ -3510,7 +3500,7 @@
       </c>
       <c r="F18" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="6" t="s">
         <v>803</v>
       </c>
@@ -3520,7 +3510,7 @@
       <c r="C19" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="45" t="s">
+      <c r="D19" s="43" t="s">
         <v>838</v>
       </c>
       <c r="E19" s="25" t="s">
@@ -3528,7 +3518,7 @@
       </c>
       <c r="F19" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="6" t="s">
         <v>803</v>
       </c>
@@ -7234,7 +7224,7 @@
     <col min="6" max="6" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -7254,7 +7244,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="6" t="s">
         <v>276</v>
       </c>
@@ -7274,7 +7264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="6" t="s">
         <v>276</v>
       </c>
@@ -7294,7 +7284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="6" t="s">
         <v>276</v>
       </c>
@@ -7314,7 +7304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="6" t="s">
         <v>276</v>
       </c>
@@ -7334,7 +7324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="6" t="s">
         <v>276</v>
       </c>
@@ -7354,7 +7344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="6" t="s">
         <v>276</v>
       </c>
@@ -7374,7 +7364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="6" t="s">
         <v>276</v>
       </c>
@@ -7394,7 +7384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="6" t="s">
         <v>276</v>
       </c>
@@ -7414,7 +7404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="6" t="s">
         <v>276</v>
       </c>
@@ -7434,7 +7424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="6" t="s">
         <v>276</v>
       </c>
@@ -7454,7 +7444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="6" t="s">
         <v>276</v>
       </c>
@@ -7474,7 +7464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="6" t="s">
         <v>276</v>
       </c>
@@ -7494,7 +7484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="6" t="s">
         <v>276</v>
       </c>
@@ -7514,7 +7504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="6" t="s">
         <v>276</v>
       </c>
@@ -7534,7 +7524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="6" t="s">
         <v>276</v>
       </c>
@@ -7554,7 +7544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="6" t="s">
         <v>276</v>
       </c>
@@ -7574,7 +7564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="6" t="s">
         <v>276</v>
       </c>
@@ -7594,7 +7584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="6" t="s">
         <v>276</v>
       </c>
@@ -10943,7 +10933,7 @@
       <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="43" t="s">
+      <c r="F1" s="41" t="s">
         <v>5</v>
       </c>
     </row>
@@ -11686,7 +11676,7 @@
       <c r="B9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="44" t="s">
+      <c r="C9" s="42" t="s">
         <v>786</v>
       </c>
       <c r="D9" s="14" t="s">
@@ -11757,7 +11747,7 @@
       <c r="D1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="43" t="s">
+      <c r="E1" s="41" t="s">
         <v>5</v>
       </c>
     </row>
@@ -12440,274 +12430,274 @@
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="36" t="s">
+      <c r="A1" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="36" t="s">
+      <c r="C1" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="36" t="s">
+      <c r="D1" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="36" t="s">
+      <c r="E1" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="37" t="s">
+      <c r="F1" s="35" t="s">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="37" t="s">
         <v>748</v>
       </c>
-      <c r="C2" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="39" t="s">
+      <c r="C2" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="39" t="s">
+      <c r="E2" s="37" t="s">
         <v>749</v>
       </c>
-      <c r="F2" s="40">
+      <c r="F2" s="38">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="37" t="s">
         <v>750</v>
       </c>
-      <c r="C3" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="39" t="s">
+      <c r="C3" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="39" t="s">
+      <c r="E3" s="37" t="s">
         <v>751</v>
       </c>
-      <c r="F3" s="40">
+      <c r="F3" s="38">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B4" s="39" t="s">
+      <c r="B4" s="37" t="s">
         <v>752</v>
       </c>
-      <c r="C4" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="39" t="s">
+      <c r="C4" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="37" t="s">
         <v>753</v>
       </c>
-      <c r="E4" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="41"/>
+      <c r="E4" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="39"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="37" t="s">
         <v>754</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="D5" s="39" t="s">
+      <c r="D5" s="37" t="s">
         <v>755</v>
       </c>
-      <c r="E5" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="40">
+      <c r="E5" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="38">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="38" t="s">
+      <c r="A6" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="37" t="s">
         <v>756</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D6" s="37" t="s">
         <v>757</v>
       </c>
-      <c r="E6" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="40">
+      <c r="E6" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="38">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="38" t="s">
+      <c r="A7" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="37" t="s">
         <v>758</v>
       </c>
-      <c r="C7" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="39" t="s">
+      <c r="C7" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="37" t="s">
         <v>759</v>
       </c>
-      <c r="E7" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="41"/>
+      <c r="E7" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="39"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="37" t="s">
         <v>760</v>
       </c>
-      <c r="C8" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="39" t="s">
+      <c r="C8" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="37" t="s">
         <v>761</v>
       </c>
-      <c r="E8" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="41"/>
+      <c r="E8" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="39"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="38" t="s">
+      <c r="A9" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="37" t="s">
         <v>762</v>
       </c>
-      <c r="C9" s="39" t="s">
+      <c r="C9" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="D9" s="39" t="s">
+      <c r="D9" s="37" t="s">
         <v>763</v>
       </c>
-      <c r="E9" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" s="40">
+      <c r="E9" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="38">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="38" t="s">
+      <c r="A10" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B10" s="39" t="s">
+      <c r="B10" s="37" t="s">
         <v>764</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="39" t="s">
+      <c r="D10" s="37" t="s">
         <v>765</v>
       </c>
-      <c r="E10" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="40">
+      <c r="E10" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="38">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="38" t="s">
+      <c r="A11" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B11" s="39" t="s">
+      <c r="B11" s="37" t="s">
         <v>488</v>
       </c>
-      <c r="C11" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="39" t="s">
+      <c r="C11" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="37" t="s">
         <v>766</v>
       </c>
-      <c r="E11" s="39" t="s">
+      <c r="E11" s="37" t="s">
         <v>489</v>
       </c>
-      <c r="F11" s="40">
+      <c r="F11" s="38">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B12" s="39" t="s">
+      <c r="B12" s="37" t="s">
         <v>490</v>
       </c>
-      <c r="C12" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="39" t="s">
+      <c r="C12" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="37" t="s">
         <v>766</v>
       </c>
-      <c r="E12" s="39" t="s">
+      <c r="E12" s="37" t="s">
         <v>491</v>
       </c>
-      <c r="F12" s="40">
+      <c r="F12" s="38">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="38" t="s">
+      <c r="A13" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="37" t="s">
         <v>767</v>
       </c>
-      <c r="C13" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="39" t="s">
+      <c r="C13" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="37" t="s">
         <v>768</v>
       </c>
-      <c r="E13" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" s="41"/>
+      <c r="E13" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" s="39"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="38" t="s">
+      <c r="A14" s="36" t="s">
         <v>747</v>
       </c>
-      <c r="B14" s="38" t="s">
+      <c r="B14" s="36" t="s">
         <v>769</v>
       </c>
-      <c r="C14" s="38" t="s">
+      <c r="C14" s="36" t="s">
         <v>68</v>
       </c>
-      <c r="D14" s="38" t="s">
+      <c r="D14" s="36" t="s">
         <v>770</v>
       </c>
-      <c r="E14" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="42">
+      <c r="E14" s="36" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="40">
         <v>0</v>
       </c>
     </row>
@@ -13096,33 +13086,35 @@
       <c r="A20" s="17" t="s">
         <v>643</v>
       </c>
-      <c r="B20" s="33" t="s">
+      <c r="B20" s="25" t="s">
         <v>661</v>
       </c>
       <c r="C20" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="D20" s="34" t="s">
+      <c r="D20" s="7" t="s">
         <v>662</v>
       </c>
-      <c r="E20" s="33"/>
-      <c r="F20" s="34"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="17" t="s">
         <v>643</v>
       </c>
-      <c r="B21" s="33" t="s">
+      <c r="B21" s="25" t="s">
         <v>663</v>
       </c>
       <c r="C21" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="D21" s="34" t="s">
+      <c r="D21" s="7" t="s">
         <v>664</v>
       </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="34"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="7">
+        <v>0</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="17" t="s">
@@ -13132,15 +13124,17 @@
         <v>665</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="D22" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="E22" s="17" t="s">
         <v>666</v>
       </c>
-      <c r="E22" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="F22" s="18"/>
+      <c r="F22" s="18">
+        <v>0</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="17" t="s">
@@ -13150,17 +13144,15 @@
         <v>667</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="D23" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="E23" s="17" t="s">
         <v>668</v>
       </c>
-      <c r="E23" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="F23" s="18">
-        <v>0</v>
-      </c>
+      <c r="F23" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="17" t="s">
@@ -13518,7 +13510,7 @@
         <v>697</v>
       </c>
       <c r="C43" s="17" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="D43" s="32" t="s">
         <v>698</v>
@@ -13526,9 +13518,7 @@
       <c r="E43" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F43" s="16">
-        <v>0</v>
-      </c>
+      <c r="F43" s="16"/>
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
       <c r="A44" s="17" t="s">

</xml_diff>

<commit_message>
added gamimngLobby for GH and NG
</commit_message>
<xml_diff>
--- a/src/global/utils/file-utils/locators(2).xlsx
+++ b/src/global/utils/file-utils/locators(2).xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="17"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="HomePage"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2917" uniqueCount="841">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2992" uniqueCount="856">
   <si>
     <t>page</t>
   </si>
@@ -1828,13 +1828,16 @@
     <t>:text("Results") &gt;&gt; svg</t>
   </si>
   <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
     <t>GamingLobbyPage</t>
   </si>
   <si>
     <t>Aviator</t>
   </si>
   <si>
-    <t>a[href='/lobby/casino-games/game/aviator']</t>
+    <t>a[href='/lobby/Casino/featured/Aviator']</t>
   </si>
   <si>
     <t>loginInPopup</t>
@@ -1876,16 +1879,25 @@
     <t>casinoGames</t>
   </si>
   <si>
-    <t>casino games</t>
-  </si>
-  <si>
     <t>{ "hasText": true }</t>
   </si>
   <si>
     <t>promotionsInCasino</t>
   </si>
   <si>
-    <t>//img[@alt='/Betway/South-Africa/SA_Responsible_gambling_CL/']</t>
+    <t>//img[@alt='/Betway/South-Africa/SA_Hacksaw_LeBandit_DeulAtDawn_NewGames/']</t>
+  </si>
+  <si>
+    <t>promotionsInCasinoNG</t>
+  </si>
+  <si>
+    <t>//img[@alt='/Betway/Nigeria/NG_Premier_League_Reels/']</t>
+  </si>
+  <si>
+    <t>promotionsInCasinoGH</t>
+  </si>
+  <si>
+    <t>//img[@alt='/Betway/Ghana/GH_Drops_and_Wins_26/']</t>
   </si>
   <si>
     <t>casinoSearch</t>
@@ -1918,18 +1930,36 @@
     <t>betGames</t>
   </si>
   <si>
+    <t>a[href='/lobby/betgames']</t>
+  </si>
+  <si>
+    <t>promotionsInBetGamesNG</t>
+  </si>
+  <si>
+    <t>img</t>
+  </si>
+  <si>
+    <t>{"name": "/Betway/Nigeria-Synapse/NG_Betgames_New_Lobby_Lucky7/"}</t>
+  </si>
+  <si>
+    <t>promotionsInBetGamesGH</t>
+  </si>
+  <si>
+    <t>{ "name": "/Betway/Ghana/Betgames_New_Lobby_Lucky7/" }</t>
+  </si>
+  <si>
     <t>promotionsInBetGames</t>
   </si>
   <si>
-    <t>img</t>
-  </si>
-  <si>
     <t>{ "name": "/Betway/South-Africa/Betgames_New_Lobby_Skyward/" }</t>
   </si>
   <si>
     <t>betGamesFilter</t>
   </si>
   <si>
+    <t>a[href='/lobby/betgames/betgames'].flex.gap-2.items-center</t>
+  </si>
+  <si>
     <t>gameDivBetGames</t>
   </si>
   <si>
@@ -1939,6 +1969,18 @@
     <t>virtuals</t>
   </si>
   <si>
+    <t>promotionsInVirtualsNG</t>
+  </si>
+  <si>
+    <t>{ "name": "/Betway/Nigeria-Synapse/Virtuals-_New_Lobby_PlatHounds/" }</t>
+  </si>
+  <si>
+    <t>promotionsInVirtualsGH</t>
+  </si>
+  <si>
+    <t>{ "name": "/Betway/Ghana/GH_FansWorldCup/" }</t>
+  </si>
+  <si>
     <t>promotionsInVirtuals</t>
   </si>
   <si>
@@ -1964,6 +2006,9 @@
   </si>
   <si>
     <t>//*[@id="tab"]/div/div[3]/div/div[2]/div/div/div[1]/div[1]</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>HeaderPage</t>
@@ -2729,7 +2774,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="50">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2825,6 +2870,21 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="12" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
@@ -3192,16 +3252,16 @@
       <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="42" t="s">
+      <c r="F1" s="47" t="s">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>805</v>
+        <v>820</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>8</v>
@@ -3210,7 +3270,7 @@
         <v>30</v>
       </c>
       <c r="E2" s="26" t="s">
-        <v>806</v>
+        <v>821</v>
       </c>
       <c r="F2" s="8">
         <v>1</v>
@@ -3218,10 +3278,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>807</v>
+        <v>822</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>8</v>
@@ -3230,22 +3290,22 @@
         <v>30</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>808</v>
+        <v>823</v>
       </c>
       <c r="F3" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>809</v>
+        <v>824</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>810</v>
+        <v>825</v>
       </c>
       <c r="E4" s="26" t="s">
         <v>23</v>
@@ -3254,10 +3314,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>811</v>
+        <v>826</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>8</v>
@@ -3266,16 +3326,16 @@
         <v>30</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>812</v>
+        <v>827</v>
       </c>
       <c r="F5" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>813</v>
+        <v>828</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>8</v>
@@ -3284,16 +3344,16 @@
         <v>30</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>814</v>
+        <v>829</v>
       </c>
       <c r="F6" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>815</v>
+        <v>830</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>8</v>
@@ -3302,22 +3362,22 @@
         <v>30</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>816</v>
+        <v>831</v>
       </c>
       <c r="F7" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>817</v>
+        <v>832</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>818</v>
+        <v>833</v>
       </c>
       <c r="E8" s="26" t="s">
         <v>23</v>
@@ -3326,16 +3386,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>819</v>
+        <v>834</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>820</v>
+        <v>835</v>
       </c>
       <c r="E9" s="26" t="s">
         <v>23</v>
@@ -3344,16 +3404,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>821</v>
+        <v>836</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>822</v>
+        <v>837</v>
       </c>
       <c r="E10" s="26" t="s">
         <v>23</v>
@@ -3362,10 +3422,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>823</v>
+        <v>838</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>8</v>
@@ -3374,7 +3434,7 @@
         <v>30</v>
       </c>
       <c r="E11" s="26" t="s">
-        <v>824</v>
+        <v>839</v>
       </c>
       <c r="F11" s="8">
         <v>0</v>
@@ -3382,16 +3442,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>825</v>
+        <v>840</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>826</v>
+        <v>841</v>
       </c>
       <c r="E12" s="26" t="s">
         <v>23</v>
@@ -3400,16 +3460,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>827</v>
+        <v>842</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>827</v>
+        <v>842</v>
       </c>
       <c r="E13" s="26" t="s">
         <v>23</v>
@@ -3418,16 +3478,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>828</v>
+        <v>843</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>829</v>
+        <v>844</v>
       </c>
       <c r="E14" s="26" t="s">
         <v>23</v>
@@ -3436,16 +3496,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>830</v>
+        <v>845</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>831</v>
+        <v>846</v>
       </c>
       <c r="E15" s="26" t="s">
         <v>23</v>
@@ -3454,16 +3514,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>832</v>
+        <v>847</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>833</v>
+        <v>848</v>
       </c>
       <c r="E16" s="26" t="s">
         <v>23</v>
@@ -3472,16 +3532,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>834</v>
+        <v>849</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>835</v>
+        <v>850</v>
       </c>
       <c r="E17" s="26" t="s">
         <v>23</v>
@@ -3490,16 +3550,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>836</v>
+        <v>851</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>837</v>
+        <v>852</v>
       </c>
       <c r="E18" s="26" t="s">
         <v>23</v>
@@ -3508,16 +3568,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>838</v>
+        <v>853</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="44" t="s">
-        <v>839</v>
+      <c r="D19" s="49" t="s">
+        <v>854</v>
       </c>
       <c r="E19" s="26" t="s">
         <v>23</v>
@@ -3526,10 +3586,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="6" t="s">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>840</v>
+        <v>855</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>8</v>
@@ -3538,7 +3598,7 @@
         <v>30</v>
       </c>
       <c r="E20" s="26" t="s">
-        <v>806</v>
+        <v>821</v>
       </c>
       <c r="F20" s="8"/>
     </row>
@@ -10961,13 +11021,13 @@
       <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="42" t="s">
+      <c r="F1" s="47" t="s">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>178</v>
@@ -10987,7 +11047,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>189</v>
@@ -10999,7 +11059,7 @@
         <v>30</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>794</v>
+        <v>809</v>
       </c>
       <c r="F3" s="8">
         <v>0</v>
@@ -11007,7 +11067,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>191</v>
@@ -11027,7 +11087,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>193</v>
@@ -11047,7 +11107,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>195</v>
@@ -11067,7 +11127,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>197</v>
@@ -11087,7 +11147,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>199</v>
@@ -11099,7 +11159,7 @@
         <v>30</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>795</v>
+        <v>810</v>
       </c>
       <c r="F8" s="8">
         <v>0</v>
@@ -11107,7 +11167,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>201</v>
@@ -11119,7 +11179,7 @@
         <v>30</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>796</v>
+        <v>811</v>
       </c>
       <c r="F9" s="8">
         <v>0</v>
@@ -11127,7 +11187,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>203</v>
@@ -11139,7 +11199,7 @@
         <v>30</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>797</v>
+        <v>812</v>
       </c>
       <c r="F10" s="8">
         <v>0</v>
@@ -11147,7 +11207,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>205</v>
@@ -11159,7 +11219,7 @@
         <v>30</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>798</v>
+        <v>813</v>
       </c>
       <c r="F11" s="8">
         <v>0</v>
@@ -11167,7 +11227,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>207</v>
@@ -11179,7 +11239,7 @@
         <v>30</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>799</v>
+        <v>814</v>
       </c>
       <c r="F12" s="8">
         <v>0</v>
@@ -11187,7 +11247,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>209</v>
@@ -11199,7 +11259,7 @@
         <v>30</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>800</v>
+        <v>815</v>
       </c>
       <c r="F13" s="8">
         <v>0</v>
@@ -11207,7 +11267,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>211</v>
@@ -11227,7 +11287,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>213</v>
@@ -11239,7 +11299,7 @@
         <v>30</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>801</v>
+        <v>816</v>
       </c>
       <c r="F15" s="8">
         <v>0</v>
@@ -11247,7 +11307,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>215</v>
@@ -11259,7 +11319,7 @@
         <v>30</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>802</v>
+        <v>817</v>
       </c>
       <c r="F16" s="8">
         <v>0</v>
@@ -11267,7 +11327,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>217</v>
@@ -11279,7 +11339,7 @@
         <v>30</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="F17" s="8">
         <v>0</v>
@@ -11287,7 +11347,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>219</v>
@@ -11307,7 +11367,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>384</v>
@@ -11327,7 +11387,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>222</v>
@@ -11347,7 +11407,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>223</v>
@@ -11367,7 +11427,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>32</v>
@@ -11387,7 +11447,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>225</v>
@@ -11407,7 +11467,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>227</v>
@@ -11427,7 +11487,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>229</v>
@@ -11447,7 +11507,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="6" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>231</v>
@@ -11544,7 +11604,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>792</v>
+        <v>807</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>23</v>
@@ -11592,13 +11652,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="15" t="s">
-        <v>773</v>
+        <v>788</v>
       </c>
       <c r="B2" s="15" t="s">
         <v>68</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>774</v>
+        <v>789</v>
       </c>
       <c r="D2" s="15" t="s">
         <v>23</v>
@@ -11609,13 +11669,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="15" t="s">
-        <v>775</v>
+        <v>790</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>68</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>776</v>
+        <v>791</v>
       </c>
       <c r="D3" s="15" t="s">
         <v>23</v>
@@ -11624,13 +11684,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="15" t="s">
-        <v>777</v>
+        <v>792</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>68</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>778</v>
+        <v>793</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>23</v>
@@ -11639,13 +11699,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="15" t="s">
-        <v>779</v>
+        <v>794</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>68</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>780</v>
+        <v>795</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>23</v>
@@ -11654,13 +11714,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="15" t="s">
-        <v>781</v>
+        <v>796</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>68</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>782</v>
+        <v>797</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>23</v>
@@ -11675,7 +11735,7 @@
         <v>21</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>783</v>
+        <v>798</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>23</v>
@@ -11684,13 +11744,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="6" t="s">
-        <v>784</v>
+        <v>799</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>785</v>
+        <v>800</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>23</v>
@@ -11699,13 +11759,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="6" t="s">
-        <v>786</v>
+        <v>801</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="43" t="s">
-        <v>787</v>
+      <c r="C9" s="48" t="s">
+        <v>802</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>23</v>
@@ -11714,13 +11774,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="6" t="s">
-        <v>788</v>
+        <v>803</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>68</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>789</v>
+        <v>804</v>
       </c>
       <c r="D10" s="15" t="s">
         <v>23</v>
@@ -11729,7 +11789,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="6" t="s">
-        <v>790</v>
+        <v>805</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>8</v>
@@ -11738,7 +11798,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>791</v>
+        <v>806</v>
       </c>
       <c r="E11" s="8"/>
     </row>
@@ -11775,7 +11835,7 @@
       <c r="D1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="42" t="s">
+      <c r="E1" s="47" t="s">
         <v>5</v>
       </c>
     </row>
@@ -11807,7 +11867,7 @@
         <v>9</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>772</v>
+        <v>787</v>
       </c>
       <c r="E3" s="16">
         <v>0</v>
@@ -12458,274 +12518,274 @@
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="34" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="35" t="s">
+      <c r="A1" s="39" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="E1" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="36" t="s">
+      <c r="F1" s="41" t="s">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B2" s="38" t="s">
-        <v>749</v>
-      </c>
-      <c r="C2" s="38" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="38" t="s">
+      <c r="A2" s="42" t="s">
+        <v>763</v>
+      </c>
+      <c r="B2" s="43" t="s">
+        <v>764</v>
+      </c>
+      <c r="C2" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="38" t="s">
-        <v>750</v>
-      </c>
-      <c r="F2" s="39">
+      <c r="E2" s="43" t="s">
+        <v>765</v>
+      </c>
+      <c r="F2" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B3" s="38" t="s">
-        <v>751</v>
-      </c>
-      <c r="C3" s="38" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="38" t="s">
+      <c r="A3" s="42" t="s">
+        <v>763</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>766</v>
+      </c>
+      <c r="C3" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="38" t="s">
-        <v>752</v>
-      </c>
-      <c r="F3" s="39">
+      <c r="E3" s="43" t="s">
+        <v>767</v>
+      </c>
+      <c r="F3" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B4" s="38" t="s">
-        <v>753</v>
-      </c>
-      <c r="C4" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="38" t="s">
-        <v>754</v>
-      </c>
-      <c r="E4" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="40"/>
+      <c r="A4" s="42" t="s">
+        <v>763</v>
+      </c>
+      <c r="B4" s="43" t="s">
+        <v>768</v>
+      </c>
+      <c r="C4" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="43" t="s">
+        <v>769</v>
+      </c>
+      <c r="E4" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="45"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B5" s="38" t="s">
-        <v>755</v>
-      </c>
-      <c r="C5" s="38" t="s">
+      <c r="A5" s="42" t="s">
+        <v>763</v>
+      </c>
+      <c r="B5" s="43" t="s">
+        <v>770</v>
+      </c>
+      <c r="C5" s="43" t="s">
         <v>68</v>
       </c>
-      <c r="D5" s="38" t="s">
-        <v>756</v>
-      </c>
-      <c r="E5" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="39">
+      <c r="D5" s="43" t="s">
+        <v>771</v>
+      </c>
+      <c r="E5" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B6" s="38" t="s">
-        <v>757</v>
-      </c>
-      <c r="C6" s="38" t="s">
+      <c r="A6" s="42" t="s">
+        <v>763</v>
+      </c>
+      <c r="B6" s="43" t="s">
+        <v>772</v>
+      </c>
+      <c r="C6" s="43" t="s">
         <v>68</v>
       </c>
-      <c r="D6" s="38" t="s">
-        <v>758</v>
-      </c>
-      <c r="E6" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="39">
+      <c r="D6" s="43" t="s">
+        <v>773</v>
+      </c>
+      <c r="E6" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B7" s="38" t="s">
-        <v>759</v>
-      </c>
-      <c r="C7" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="38" t="s">
-        <v>760</v>
-      </c>
-      <c r="E7" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="40"/>
+      <c r="A7" s="42" t="s">
+        <v>763</v>
+      </c>
+      <c r="B7" s="43" t="s">
+        <v>774</v>
+      </c>
+      <c r="C7" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="43" t="s">
+        <v>775</v>
+      </c>
+      <c r="E7" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="45"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B8" s="38" t="s">
-        <v>761</v>
-      </c>
-      <c r="C8" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="38" t="s">
-        <v>762</v>
-      </c>
-      <c r="E8" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="40"/>
+      <c r="A8" s="42" t="s">
+        <v>763</v>
+      </c>
+      <c r="B8" s="43" t="s">
+        <v>776</v>
+      </c>
+      <c r="C8" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>777</v>
+      </c>
+      <c r="E8" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="45"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B9" s="38" t="s">
+      <c r="A9" s="42" t="s">
         <v>763</v>
       </c>
-      <c r="C9" s="38" t="s">
+      <c r="B9" s="43" t="s">
+        <v>778</v>
+      </c>
+      <c r="C9" s="43" t="s">
         <v>68</v>
       </c>
-      <c r="D9" s="38" t="s">
-        <v>764</v>
-      </c>
-      <c r="E9" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" s="39">
+      <c r="D9" s="43" t="s">
+        <v>779</v>
+      </c>
+      <c r="E9" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B10" s="38" t="s">
-        <v>765</v>
-      </c>
-      <c r="C10" s="38" t="s">
+      <c r="A10" s="42" t="s">
+        <v>763</v>
+      </c>
+      <c r="B10" s="43" t="s">
+        <v>780</v>
+      </c>
+      <c r="C10" s="43" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="38" t="s">
-        <v>766</v>
-      </c>
-      <c r="E10" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="39">
+      <c r="D10" s="43" t="s">
+        <v>781</v>
+      </c>
+      <c r="E10" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B11" s="38" t="s">
+      <c r="A11" s="42" t="s">
+        <v>763</v>
+      </c>
+      <c r="B11" s="43" t="s">
         <v>489</v>
       </c>
-      <c r="C11" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="38" t="s">
-        <v>767</v>
-      </c>
-      <c r="E11" s="38" t="s">
+      <c r="C11" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="43" t="s">
+        <v>782</v>
+      </c>
+      <c r="E11" s="43" t="s">
         <v>490</v>
       </c>
-      <c r="F11" s="39">
+      <c r="F11" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B12" s="38" t="s">
+      <c r="A12" s="42" t="s">
+        <v>763</v>
+      </c>
+      <c r="B12" s="43" t="s">
         <v>491</v>
       </c>
-      <c r="C12" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="38" t="s">
-        <v>767</v>
-      </c>
-      <c r="E12" s="38" t="s">
+      <c r="C12" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="43" t="s">
+        <v>782</v>
+      </c>
+      <c r="E12" s="43" t="s">
         <v>492</v>
       </c>
-      <c r="F12" s="39">
+      <c r="F12" s="44">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B13" s="38" t="s">
-        <v>768</v>
-      </c>
-      <c r="C13" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="38" t="s">
-        <v>769</v>
-      </c>
-      <c r="E13" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" s="40"/>
+      <c r="A13" s="42" t="s">
+        <v>763</v>
+      </c>
+      <c r="B13" s="43" t="s">
+        <v>783</v>
+      </c>
+      <c r="C13" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="43" t="s">
+        <v>784</v>
+      </c>
+      <c r="E13" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" s="45"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="37" t="s">
-        <v>748</v>
-      </c>
-      <c r="B14" s="37" t="s">
-        <v>770</v>
-      </c>
-      <c r="C14" s="37" t="s">
+      <c r="A14" s="42" t="s">
+        <v>763</v>
+      </c>
+      <c r="B14" s="42" t="s">
+        <v>785</v>
+      </c>
+      <c r="C14" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="D14" s="37" t="s">
-        <v>771</v>
-      </c>
-      <c r="E14" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="41">
+      <c r="D14" s="42" t="s">
+        <v>786</v>
+      </c>
+      <c r="E14" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="46">
         <v>0</v>
       </c>
     </row>
@@ -12772,19 +12832,19 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>645</v>
+        <v>660</v>
       </c>
       <c r="C2" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="33" t="s">
+      <c r="D2" s="38" t="s">
         <v>30</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>646</v>
+        <v>661</v>
       </c>
       <c r="F2" s="19">
         <v>0</v>
@@ -12792,7 +12852,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B3" s="18" t="s">
         <v>7</v>
@@ -12800,7 +12860,7 @@
       <c r="C3" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="33" t="s">
+      <c r="D3" s="38" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="18" t="s">
@@ -12810,7 +12870,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>273</v>
@@ -12818,7 +12878,7 @@
       <c r="C4" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="D4" s="38" t="s">
         <v>274</v>
       </c>
       <c r="E4" s="18" t="s">
@@ -12828,7 +12888,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>275</v>
@@ -12836,7 +12896,7 @@
       <c r="C5" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="38" t="s">
         <v>77</v>
       </c>
       <c r="E5" s="18" t="s">
@@ -12848,7 +12908,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B6" s="18" t="s">
         <v>105</v>
@@ -12856,7 +12916,7 @@
       <c r="C6" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="33" t="s">
+      <c r="D6" s="38" t="s">
         <v>106</v>
       </c>
       <c r="E6" s="18" t="s">
@@ -12866,7 +12926,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B7" s="18" t="s">
         <v>13</v>
@@ -12874,7 +12934,7 @@
       <c r="C7" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="33" t="s">
+      <c r="D7" s="38" t="s">
         <v>171</v>
       </c>
       <c r="E7" s="18" t="s">
@@ -12884,7 +12944,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B8" s="18" t="s">
         <v>172</v>
@@ -12892,7 +12952,7 @@
       <c r="C8" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="33" t="s">
+      <c r="D8" s="38" t="s">
         <v>14</v>
       </c>
       <c r="E8" s="18" t="s">
@@ -12904,15 +12964,15 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>647</v>
+        <v>662</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="38" t="s">
         <v>14</v>
       </c>
       <c r="E9" s="18" t="s">
@@ -12924,7 +12984,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B10" s="18" t="s">
         <v>174</v>
@@ -12932,7 +12992,7 @@
       <c r="C10" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="33" t="s">
+      <c r="D10" s="38" t="s">
         <v>14</v>
       </c>
       <c r="E10" s="18" t="s">
@@ -12942,7 +13002,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B11" s="18" t="s">
         <v>176</v>
@@ -12950,7 +13010,7 @@
       <c r="C11" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="33" t="s">
+      <c r="D11" s="38" t="s">
         <v>14</v>
       </c>
       <c r="E11" s="18" t="s">
@@ -12962,16 +13022,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>648</v>
+        <v>663</v>
       </c>
       <c r="C12" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="33" t="s">
-        <v>649</v>
+      <c r="D12" s="38" t="s">
+        <v>664</v>
       </c>
       <c r="E12" s="18" t="s">
         <v>23</v>
@@ -12980,16 +13040,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>650</v>
+        <v>665</v>
       </c>
       <c r="C13" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="33" t="s">
-        <v>651</v>
+      <c r="D13" s="38" t="s">
+        <v>666</v>
       </c>
       <c r="E13" s="18" t="s">
         <v>23</v>
@@ -13000,16 +13060,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>652</v>
+        <v>667</v>
       </c>
       <c r="C14" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="33" t="s">
-        <v>653</v>
+      <c r="D14" s="38" t="s">
+        <v>668</v>
       </c>
       <c r="E14" s="18" t="s">
         <v>23</v>
@@ -13020,16 +13080,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>654</v>
+        <v>669</v>
       </c>
       <c r="C15" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D15" s="33" t="s">
-        <v>655</v>
+      <c r="D15" s="38" t="s">
+        <v>670</v>
       </c>
       <c r="E15" s="18" t="s">
         <v>23</v>
@@ -13038,16 +13098,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>656</v>
+        <v>671</v>
       </c>
       <c r="C16" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D16" s="33" t="s">
-        <v>657</v>
+      <c r="D16" s="38" t="s">
+        <v>672</v>
       </c>
       <c r="E16" s="18" t="s">
         <v>23</v>
@@ -13056,16 +13116,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>658</v>
+        <v>673</v>
       </c>
       <c r="C17" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D17" s="33" t="s">
-        <v>655</v>
+      <c r="D17" s="38" t="s">
+        <v>670</v>
       </c>
       <c r="E17" s="18" t="s">
         <v>23</v>
@@ -13074,16 +13134,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>659</v>
+        <v>674</v>
       </c>
       <c r="C18" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="33" t="s">
-        <v>657</v>
+      <c r="D18" s="38" t="s">
+        <v>672</v>
       </c>
       <c r="E18" s="18" t="s">
         <v>23</v>
@@ -13094,16 +13154,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>660</v>
+        <v>675</v>
       </c>
       <c r="C19" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D19" s="33" t="s">
-        <v>661</v>
+      <c r="D19" s="38" t="s">
+        <v>676</v>
       </c>
       <c r="E19" s="18" t="s">
         <v>23</v>
@@ -13112,32 +13172,32 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>662</v>
+        <v>677</v>
       </c>
       <c r="C20" s="18" t="s">
         <v>68</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>663</v>
+        <v>678</v>
       </c>
       <c r="E20" s="26"/>
       <c r="F20" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>664</v>
+        <v>679</v>
       </c>
       <c r="C21" s="18" t="s">
         <v>68</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>665</v>
+        <v>680</v>
       </c>
       <c r="E21" s="26"/>
       <c r="F21" s="7">
@@ -13146,19 +13206,19 @@
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="C22" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="33" t="s">
+      <c r="D22" s="38" t="s">
         <v>30</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>667</v>
+        <v>682</v>
       </c>
       <c r="F22" s="19">
         <v>0</v>
@@ -13166,34 +13226,34 @@
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>668</v>
+        <v>683</v>
       </c>
       <c r="C23" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D23" s="33" t="s">
+      <c r="D23" s="38" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>669</v>
+        <v>684</v>
       </c>
       <c r="F23" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="C24" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D24" s="33" t="s">
-        <v>671</v>
+      <c r="D24" s="38" t="s">
+        <v>686</v>
       </c>
       <c r="E24" s="18" t="s">
         <v>23</v>
@@ -13202,10 +13262,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="C25" s="18" t="s">
         <v>68</v>
@@ -13222,15 +13282,15 @@
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
       <c r="C26" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D26" s="33" t="s">
+      <c r="D26" s="38" t="s">
         <v>381</v>
       </c>
       <c r="E26" s="18" t="s">
@@ -13240,7 +13300,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B27" s="18" t="s">
         <v>167</v>
@@ -13248,7 +13308,7 @@
       <c r="C27" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D27" s="33" t="s">
+      <c r="D27" s="38" t="s">
         <v>382</v>
       </c>
       <c r="E27" s="18" t="s">
@@ -13258,16 +13318,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>674</v>
+        <v>689</v>
       </c>
       <c r="C28" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="33" t="s">
-        <v>675</v>
+      <c r="D28" s="38" t="s">
+        <v>690</v>
       </c>
       <c r="E28" s="18" t="s">
         <v>23</v>
@@ -13276,16 +13336,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
       <c r="A29" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
       <c r="C29" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D29" s="33" t="s">
-        <v>677</v>
+      <c r="D29" s="38" t="s">
+        <v>692</v>
       </c>
       <c r="E29" s="18" t="s">
         <v>23</v>
@@ -13294,7 +13354,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B30" s="18" t="s">
         <v>384</v>
@@ -13302,7 +13362,7 @@
       <c r="C30" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D30" s="33" t="s">
+      <c r="D30" s="38" t="s">
         <v>385</v>
       </c>
       <c r="E30" s="18" t="s">
@@ -13312,15 +13372,15 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>678</v>
+        <v>693</v>
       </c>
       <c r="C31" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D31" s="33" t="s">
+      <c r="D31" s="38" t="s">
         <v>14</v>
       </c>
       <c r="E31" s="18" t="s">
@@ -13330,19 +13390,19 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>679</v>
+        <v>694</v>
       </c>
       <c r="C32" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D32" s="33" t="s">
+      <c r="D32" s="38" t="s">
         <v>14</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>680</v>
+        <v>695</v>
       </c>
       <c r="F32" s="17">
         <v>1</v>
@@ -13350,33 +13410,33 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>681</v>
+        <v>696</v>
       </c>
       <c r="C33" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D33" s="33" t="s">
+      <c r="D33" s="38" t="s">
         <v>14</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>682</v>
+        <v>697</v>
       </c>
       <c r="F33" s="17"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>683</v>
+        <v>698</v>
       </c>
       <c r="C34" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="33" t="s">
+      <c r="D34" s="38" t="s">
         <v>77</v>
       </c>
       <c r="E34" s="18" t="s">
@@ -13388,16 +13448,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B35" s="18" t="s">
-        <v>684</v>
+        <v>699</v>
       </c>
       <c r="C35" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D35" s="33" t="s">
-        <v>685</v>
+      <c r="D35" s="38" t="s">
+        <v>700</v>
       </c>
       <c r="E35" s="18" t="s">
         <v>23</v>
@@ -13406,16 +13466,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B36" s="18" t="s">
-        <v>686</v>
+        <v>701</v>
       </c>
       <c r="C36" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D36" s="33" t="s">
-        <v>687</v>
+      <c r="D36" s="38" t="s">
+        <v>702</v>
       </c>
       <c r="E36" s="18" t="s">
         <v>23</v>
@@ -13424,16 +13484,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
       <c r="A37" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>688</v>
+        <v>703</v>
       </c>
       <c r="C37" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D37" s="33" t="s">
-        <v>689</v>
+      <c r="D37" s="38" t="s">
+        <v>704</v>
       </c>
       <c r="E37" s="18" t="s">
         <v>23</v>
@@ -13442,16 +13502,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
       <c r="A38" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>690</v>
+        <v>705</v>
       </c>
       <c r="C38" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D38" s="33" t="s">
-        <v>691</v>
+      <c r="D38" s="38" t="s">
+        <v>706</v>
       </c>
       <c r="E38" s="18" t="s">
         <v>23</v>
@@ -13460,16 +13520,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
       <c r="A39" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>692</v>
+        <v>707</v>
       </c>
       <c r="C39" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D39" s="33" t="s">
-        <v>693</v>
+      <c r="D39" s="38" t="s">
+        <v>708</v>
       </c>
       <c r="E39" s="18" t="s">
         <v>23</v>
@@ -13478,7 +13538,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
       <c r="A40" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B40" s="18" t="s">
         <v>186</v>
@@ -13486,7 +13546,7 @@
       <c r="C40" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D40" s="33" t="s">
+      <c r="D40" s="38" t="s">
         <v>187</v>
       </c>
       <c r="E40" s="18" t="s">
@@ -13496,16 +13556,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
       <c r="A41" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>694</v>
+        <v>709</v>
       </c>
       <c r="C41" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D41" s="33" t="s">
-        <v>695</v>
+      <c r="D41" s="38" t="s">
+        <v>710</v>
       </c>
       <c r="E41" s="18" t="s">
         <v>23</v>
@@ -13514,16 +13574,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
       <c r="A42" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>696</v>
+        <v>711</v>
       </c>
       <c r="C42" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D42" s="33" t="s">
-        <v>697</v>
+      <c r="D42" s="38" t="s">
+        <v>712</v>
       </c>
       <c r="E42" s="18" t="s">
         <v>23</v>
@@ -13532,16 +13592,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
       <c r="A43" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B43" s="18" t="s">
-        <v>698</v>
+        <v>713</v>
       </c>
       <c r="C43" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D43" s="33" t="s">
-        <v>699</v>
+      <c r="D43" s="38" t="s">
+        <v>714</v>
       </c>
       <c r="E43" s="18" t="s">
         <v>23</v>
@@ -13550,16 +13610,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
       <c r="A44" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>700</v>
+        <v>715</v>
       </c>
       <c r="C44" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D44" s="33" t="s">
-        <v>701</v>
+      <c r="D44" s="38" t="s">
+        <v>716</v>
       </c>
       <c r="E44" s="18" t="s">
         <v>23</v>
@@ -13568,16 +13628,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
       <c r="A45" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>702</v>
+        <v>717</v>
       </c>
       <c r="C45" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D45" s="33" t="s">
-        <v>703</v>
+      <c r="D45" s="38" t="s">
+        <v>718</v>
       </c>
       <c r="E45" s="18" t="s">
         <v>23</v>
@@ -13586,16 +13646,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
       <c r="A46" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>704</v>
+        <v>719</v>
       </c>
       <c r="C46" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D46" s="33" t="s">
-        <v>705</v>
+      <c r="D46" s="38" t="s">
+        <v>720</v>
       </c>
       <c r="E46" s="18" t="s">
         <v>23</v>
@@ -13604,16 +13664,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
       <c r="A47" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B47" s="18" t="s">
-        <v>706</v>
+        <v>721</v>
       </c>
       <c r="C47" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D47" s="33" t="s">
-        <v>707</v>
+      <c r="D47" s="38" t="s">
+        <v>722</v>
       </c>
       <c r="E47" s="18" t="s">
         <v>23</v>
@@ -13622,16 +13682,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
       <c r="A48" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B48" s="18" t="s">
-        <v>640</v>
+        <v>654</v>
       </c>
       <c r="C48" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D48" s="33" t="s">
-        <v>641</v>
+      <c r="D48" s="38" t="s">
+        <v>655</v>
       </c>
       <c r="E48" s="18" t="s">
         <v>23</v>
@@ -13640,15 +13700,15 @@
     </row>
     <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
       <c r="A49" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B49" s="18" t="s">
-        <v>708</v>
+        <v>723</v>
       </c>
       <c r="C49" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D49" s="33" t="s">
+      <c r="D49" s="38" t="s">
         <v>77</v>
       </c>
       <c r="E49" s="18" t="s">
@@ -13660,16 +13720,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
       <c r="A50" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>709</v>
+        <v>724</v>
       </c>
       <c r="C50" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D50" s="33" t="s">
-        <v>710</v>
+      <c r="D50" s="38" t="s">
+        <v>725</v>
       </c>
       <c r="E50" s="18" t="s">
         <v>23</v>
@@ -13678,16 +13738,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
       <c r="A51" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B51" s="18" t="s">
-        <v>711</v>
+        <v>726</v>
       </c>
       <c r="C51" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D51" s="33" t="s">
-        <v>712</v>
+      <c r="D51" s="38" t="s">
+        <v>727</v>
       </c>
       <c r="E51" s="18" t="s">
         <v>23</v>
@@ -13698,16 +13758,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
       <c r="A52" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B52" s="18" t="s">
-        <v>713</v>
+        <v>728</v>
       </c>
       <c r="C52" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D52" s="33" t="s">
-        <v>714</v>
+      <c r="D52" s="38" t="s">
+        <v>729</v>
       </c>
       <c r="E52" s="18" t="s">
         <v>23</v>
@@ -13718,16 +13778,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
       <c r="A53" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B53" s="18" t="s">
-        <v>715</v>
+        <v>730</v>
       </c>
       <c r="C53" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D53" s="33" t="s">
-        <v>716</v>
+      <c r="D53" s="38" t="s">
+        <v>731</v>
       </c>
       <c r="E53" s="18" t="s">
         <v>164</v>
@@ -13736,34 +13796,34 @@
     </row>
     <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
       <c r="A54" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>717</v>
+        <v>732</v>
       </c>
       <c r="C54" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D54" s="33" t="s">
-        <v>718</v>
+      <c r="D54" s="38" t="s">
+        <v>733</v>
       </c>
       <c r="E54" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F54" s="33"/>
+      <c r="F54" s="38"/>
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
       <c r="A55" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>719</v>
+        <v>734</v>
       </c>
       <c r="C55" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D55" s="33" t="s">
-        <v>720</v>
+      <c r="D55" s="38" t="s">
+        <v>735</v>
       </c>
       <c r="E55" s="18" t="s">
         <v>23</v>
@@ -13772,16 +13832,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
       <c r="A56" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B56" s="18" t="s">
-        <v>721</v>
+        <v>736</v>
       </c>
       <c r="C56" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D56" s="33" t="s">
-        <v>722</v>
+      <c r="D56" s="38" t="s">
+        <v>737</v>
       </c>
       <c r="E56" s="18" t="s">
         <v>23</v>
@@ -13790,16 +13850,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
       <c r="A57" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B57" s="18" t="s">
-        <v>723</v>
+        <v>738</v>
       </c>
       <c r="C57" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D57" s="33" t="s">
-        <v>724</v>
+      <c r="D57" s="38" t="s">
+        <v>739</v>
       </c>
       <c r="E57" s="18" t="s">
         <v>23</v>
@@ -13808,16 +13868,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
       <c r="A58" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B58" s="18" t="s">
-        <v>725</v>
+        <v>740</v>
       </c>
       <c r="C58" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D58" s="33" t="s">
-        <v>722</v>
+      <c r="D58" s="38" t="s">
+        <v>737</v>
       </c>
       <c r="E58" s="18" t="s">
         <v>23</v>
@@ -13826,16 +13886,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
       <c r="A59" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B59" s="18" t="s">
-        <v>726</v>
+        <v>741</v>
       </c>
       <c r="C59" s="18" t="s">
-        <v>727</v>
-      </c>
-      <c r="D59" s="33" t="s">
-        <v>728</v>
+        <v>742</v>
+      </c>
+      <c r="D59" s="38" t="s">
+        <v>743</v>
       </c>
       <c r="E59" s="18" t="s">
         <v>23</v>
@@ -13844,16 +13904,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
       <c r="A60" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B60" s="18" t="s">
-        <v>729</v>
+        <v>744</v>
       </c>
       <c r="C60" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D60" s="33" t="s">
-        <v>730</v>
+      <c r="D60" s="38" t="s">
+        <v>745</v>
       </c>
       <c r="E60" s="18" t="s">
         <v>23</v>
@@ -13862,16 +13922,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
       <c r="A61" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B61" s="18" t="s">
-        <v>731</v>
+        <v>746</v>
       </c>
       <c r="C61" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D61" s="33" t="s">
-        <v>730</v>
+      <c r="D61" s="38" t="s">
+        <v>745</v>
       </c>
       <c r="E61" s="18" t="s">
         <v>23</v>
@@ -13882,16 +13942,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
       <c r="A62" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B62" s="18" t="s">
-        <v>732</v>
+        <v>747</v>
       </c>
       <c r="C62" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D62" s="33" t="s">
-        <v>722</v>
+      <c r="D62" s="38" t="s">
+        <v>737</v>
       </c>
       <c r="E62" s="18" t="s">
         <v>23</v>
@@ -13900,16 +13960,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
       <c r="A63" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B63" s="18" t="s">
-        <v>733</v>
+        <v>748</v>
       </c>
       <c r="C63" s="18" t="s">
-        <v>727</v>
-      </c>
-      <c r="D63" s="33" t="s">
-        <v>734</v>
+        <v>742</v>
+      </c>
+      <c r="D63" s="38" t="s">
+        <v>749</v>
       </c>
       <c r="E63" s="18" t="s">
         <v>23</v>
@@ -13918,19 +13978,19 @@
     </row>
     <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="19.5">
       <c r="A64" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B64" s="18" t="s">
-        <v>735</v>
+        <v>750</v>
       </c>
       <c r="C64" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D64" s="33" t="s">
+      <c r="D64" s="38" t="s">
         <v>14</v>
       </c>
       <c r="E64" s="18" t="s">
-        <v>680</v>
+        <v>695</v>
       </c>
       <c r="F64" s="19">
         <v>1</v>
@@ -13938,16 +13998,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="19.5">
       <c r="A65" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B65" s="18" t="s">
-        <v>736</v>
+        <v>751</v>
       </c>
       <c r="C65" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D65" s="33" t="s">
-        <v>737</v>
+      <c r="D65" s="38" t="s">
+        <v>752</v>
       </c>
       <c r="E65" s="18" t="s">
         <v>23</v>
@@ -13956,16 +14016,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
       <c r="A66" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B66" s="18" t="s">
-        <v>738</v>
+        <v>753</v>
       </c>
       <c r="C66" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D66" s="33" t="s">
-        <v>739</v>
+      <c r="D66" s="38" t="s">
+        <v>754</v>
       </c>
       <c r="E66" s="18" t="s">
         <v>23</v>
@@ -13974,16 +14034,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
       <c r="A67" s="26" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B67" s="26" t="s">
-        <v>740</v>
+        <v>755</v>
       </c>
       <c r="C67" s="26" t="s">
         <v>25</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>741</v>
+        <v>756</v>
       </c>
       <c r="E67" s="26" t="s">
         <v>23</v>
@@ -13992,16 +14052,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
       <c r="A68" s="26" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B68" s="26" t="s">
-        <v>742</v>
+        <v>757</v>
       </c>
       <c r="C68" s="26" t="s">
         <v>25</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>743</v>
+        <v>758</v>
       </c>
       <c r="E68" s="26" t="s">
         <v>23</v>
@@ -14010,16 +14070,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
       <c r="A69" s="26" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B69" s="26" t="s">
-        <v>744</v>
+        <v>759</v>
       </c>
       <c r="C69" s="26" t="s">
         <v>25</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>745</v>
+        <v>760</v>
       </c>
       <c r="E69" s="26" t="s">
         <v>23</v>
@@ -14028,16 +14088,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="19.5">
       <c r="A70" s="18" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="B70" s="18" t="s">
-        <v>746</v>
+        <v>761</v>
       </c>
       <c r="C70" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D70" s="33" t="s">
-        <v>747</v>
+      <c r="D70" s="38" t="s">
+        <v>762</v>
       </c>
       <c r="E70" s="18" t="s">
         <v>23</v>
@@ -14054,7 +14114,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
@@ -14082,160 +14142,172 @@
         <v>4</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>5</v>
+        <v>598</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>598</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>599</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>600</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>598</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>602</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>604</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>605</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>598</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>603</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>604</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>606</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>607</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>598</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>605</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>606</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>609</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>598</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>607</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>608</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="8"/>
+      <c r="F7" s="8" t="s">
+        <v>598</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="8">
-        <v>0</v>
+      <c r="F8" s="8" t="s">
+        <v>598</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>614</v>
+        <v>181</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>615</v>
       </c>
-      <c r="F9" s="8">
-        <v>0</v>
+      <c r="F9" s="8" t="s">
+        <v>598</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>616</v>
@@ -14249,17 +14321,19 @@
       <c r="E10" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F10" s="8"/>
+      <c r="F10" s="8" t="s">
+        <v>598</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>618</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>619</v>
@@ -14267,39 +14341,39 @@
       <c r="E11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F11" s="8">
-        <v>0</v>
+      <c r="F11" s="8" t="s">
+        <v>598</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>620</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>68</v>
+        <v>25</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>621</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>615</v>
-      </c>
-      <c r="F12" s="8">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>598</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>622</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>623</v>
@@ -14307,295 +14381,477 @@
       <c r="E13" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F13" s="8"/>
+      <c r="F13" s="8" t="s">
+        <v>598</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>321</v>
+        <v>624</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>615</v>
       </c>
-      <c r="F14" s="8">
-        <v>0</v>
+      <c r="F14" s="8" t="s">
+        <v>598</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" s="8" t="s">
         <v>598</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>625</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>626</v>
-      </c>
-      <c r="F15" s="8">
-        <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>627</v>
+        <v>321</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>199</v>
+        <v>628</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>615</v>
       </c>
-      <c r="F16" s="8"/>
+      <c r="F16" s="8" t="s">
+        <v>598</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>629</v>
+        <v>14</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>630</v>
       </c>
-      <c r="F17" s="8">
-        <v>0</v>
+      <c r="F17" s="8" t="s">
+        <v>598</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>631</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>284</v>
+        <v>632</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>615</v>
-      </c>
-      <c r="F18" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>598</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>635</v>
+      </c>
+      <c r="F19" s="8" t="s">
         <v>598</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>632</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>633</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F19" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>636</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>637</v>
+      </c>
+      <c r="F20" s="8" t="s">
         <v>598</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>634</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>615</v>
-      </c>
-      <c r="F20" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>638</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>639</v>
+      </c>
+      <c r="F21" s="8" t="s">
         <v>598</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F21" s="8">
-        <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>640</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F22" s="8" t="s">
         <v>598</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F22" s="8">
-        <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>642</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F23" s="8" t="s">
         <v>598</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F23" s="8">
-        <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>615</v>
+      </c>
+      <c r="F24" s="8" t="s">
         <v>598</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F24" s="8">
-        <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F25" s="8" t="s">
         <v>598</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>635</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>629</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>636</v>
-      </c>
-      <c r="F25" s="8">
-        <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F26" s="33" t="s">
         <v>598</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>637</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>638</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>639</v>
-      </c>
-      <c r="F26" s="8">
-        <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F27" s="33" t="s">
         <v>598</v>
       </c>
-      <c r="B27" s="18" t="s">
-        <v>640</v>
-      </c>
-      <c r="C27" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D27" s="18" t="s">
-        <v>641</v>
-      </c>
-      <c r="E27" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F27" s="17"/>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F28" s="33" t="s">
         <v>598</v>
       </c>
-      <c r="B28" s="6" t="s">
-        <v>642</v>
-      </c>
-      <c r="C28" s="6" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+      <c r="A29" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>646</v>
+      </c>
+      <c r="F29" s="33" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+      <c r="A30" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="F30" s="33" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+      <c r="A31" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>649</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>650</v>
+      </c>
+      <c r="F31" s="33" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
+      <c r="A32" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>651</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>652</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>653</v>
+      </c>
+      <c r="F32" s="33" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
+      <c r="A33" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>654</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>655</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F33" s="33" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
+      <c r="A34" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="C34" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="6" t="s">
-        <v>643</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F28" s="8"/>
+      <c r="D34" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
+      <c r="A35" s="6"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="33"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
+      <c r="A36" s="34" t="s">
+        <v>658</v>
+      </c>
+      <c r="B36" s="35" t="s">
+        <v>658</v>
+      </c>
+      <c r="C36" s="35" t="s">
+        <v>658</v>
+      </c>
+      <c r="D36" s="35" t="s">
+        <v>658</v>
+      </c>
+      <c r="E36" s="35" t="s">
+        <v>658</v>
+      </c>
+      <c r="F36" s="36" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
+      <c r="A37" s="34" t="s">
+        <v>658</v>
+      </c>
+      <c r="B37" s="34" t="s">
+        <v>658</v>
+      </c>
+      <c r="C37" s="34" t="s">
+        <v>658</v>
+      </c>
+      <c r="D37" s="34" t="s">
+        <v>658</v>
+      </c>
+      <c r="E37" s="34" t="s">
+        <v>658</v>
+      </c>
+      <c r="F37" s="37" t="s">
+        <v>658</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix Header and other scripts
</commit_message>
<xml_diff>
--- a/src/global/utils/file-utils/locators(2).xlsx
+++ b/src/global/utils/file-utils/locators(2).xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="7"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="HomePage"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2992" uniqueCount="856">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2980" uniqueCount="855">
   <si>
     <t>page</t>
   </si>
@@ -2008,9 +2008,6 @@
     <t>//*[@id="tab"]/div/div[3]/div/div[2]/div/div/div[1]/div[1]</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>HeaderPage</t>
   </si>
   <si>
@@ -2239,7 +2236,7 @@
     <t>balanceDropdown</t>
   </si>
   <si>
-    <t>//*[@id="__nuxt"]/div/div/div[1]/header/div/div[2]/div/div[2]/div[2]</t>
+    <t>//*[@id="__nuxt"]/div/div[1]/header/div/div[2]/div/div[2]/div[2]</t>
   </si>
   <si>
     <t>balanceCurrency</t>
@@ -2290,7 +2287,7 @@
     <t>notificationBellIcon</t>
   </si>
   <si>
-    <t>//*[@id="__nuxt"]/div/div[1]/div[1]/header/div/div[2]/div/div[3]</t>
+    <t>//*[@id="__nuxt"]/div/div[1]/header/div/div[2]/div/div[3]</t>
   </si>
   <si>
     <t>allBalanceTxt</t>
@@ -2607,7 +2604,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2624,6 +2621,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -2774,7 +2777,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="46">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2800,7 +2803,7 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -2809,55 +2812,49 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="12" applyFont="1" fillId="0" applyAlignment="1">
@@ -2866,61 +2863,55 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="12" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="13" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="13" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="12" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="13" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="17" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="17" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="18" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="18" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="18" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="17" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="17" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="18" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="19" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -3252,16 +3243,16 @@
       <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="47" t="s">
+      <c r="F1" s="43" t="s">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="6" t="s">
+        <v>818</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>819</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>820</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>8</v>
@@ -3270,7 +3261,7 @@
         <v>30</v>
       </c>
       <c r="E2" s="26" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="F2" s="8">
         <v>1</v>
@@ -3278,10 +3269,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>8</v>
@@ -3290,22 +3281,22 @@
         <v>30</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="F3" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="E4" s="26" t="s">
         <v>23</v>
@@ -3314,10 +3305,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>8</v>
@@ -3326,16 +3317,16 @@
         <v>30</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="F5" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>8</v>
@@ -3344,16 +3335,16 @@
         <v>30</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="F6" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>8</v>
@@ -3362,22 +3353,22 @@
         <v>30</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="F7" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="E8" s="26" t="s">
         <v>23</v>
@@ -3386,16 +3377,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="E9" s="26" t="s">
         <v>23</v>
@@ -3404,16 +3395,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="E10" s="26" t="s">
         <v>23</v>
@@ -3422,10 +3413,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>8</v>
@@ -3434,7 +3425,7 @@
         <v>30</v>
       </c>
       <c r="E11" s="26" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="F11" s="8">
         <v>0</v>
@@ -3442,16 +3433,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>839</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>840</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>841</v>
       </c>
       <c r="E12" s="26" t="s">
         <v>23</v>
@@ -3460,16 +3451,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="E13" s="26" t="s">
         <v>23</v>
@@ -3478,16 +3469,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B14" s="6" t="s">
+        <v>842</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>843</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>844</v>
       </c>
       <c r="E14" s="26" t="s">
         <v>23</v>
@@ -3496,16 +3487,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="E15" s="26" t="s">
         <v>23</v>
@@ -3514,16 +3505,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="E16" s="26" t="s">
         <v>23</v>
@@ -3532,16 +3523,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>68</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="E17" s="26" t="s">
         <v>23</v>
@@ -3550,16 +3541,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B18" s="6" t="s">
+        <v>850</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>851</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>852</v>
       </c>
       <c r="E18" s="26" t="s">
         <v>23</v>
@@ -3568,16 +3559,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B19" s="6" t="s">
+        <v>852</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D19" s="45" t="s">
         <v>853</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D19" s="49" t="s">
-        <v>854</v>
       </c>
       <c r="E19" s="26" t="s">
         <v>23</v>
@@ -3586,10 +3577,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="6" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>8</v>
@@ -3598,7 +3589,7 @@
         <v>30</v>
       </c>
       <c r="E20" s="26" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="F20" s="8"/>
     </row>
@@ -11021,13 +11012,13 @@
       <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="47" t="s">
+      <c r="F1" s="43" t="s">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>178</v>
@@ -11047,7 +11038,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>189</v>
@@ -11059,7 +11050,7 @@
         <v>30</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F3" s="8">
         <v>0</v>
@@ -11067,7 +11058,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>191</v>
@@ -11087,7 +11078,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>193</v>
@@ -11107,7 +11098,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>195</v>
@@ -11127,7 +11118,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>197</v>
@@ -11147,7 +11138,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>199</v>
@@ -11159,7 +11150,7 @@
         <v>30</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="F8" s="8">
         <v>0</v>
@@ -11167,7 +11158,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>201</v>
@@ -11179,7 +11170,7 @@
         <v>30</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="F9" s="8">
         <v>0</v>
@@ -11187,7 +11178,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>203</v>
@@ -11199,7 +11190,7 @@
         <v>30</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="F10" s="8">
         <v>0</v>
@@ -11207,7 +11198,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>205</v>
@@ -11219,7 +11210,7 @@
         <v>30</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="F11" s="8">
         <v>0</v>
@@ -11227,7 +11218,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>207</v>
@@ -11239,7 +11230,7 @@
         <v>30</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="F12" s="8">
         <v>0</v>
@@ -11247,7 +11238,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>209</v>
@@ -11259,7 +11250,7 @@
         <v>30</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="F13" s="8">
         <v>0</v>
@@ -11267,7 +11258,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>211</v>
@@ -11287,7 +11278,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>213</v>
@@ -11299,7 +11290,7 @@
         <v>30</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="F15" s="8">
         <v>0</v>
@@ -11307,7 +11298,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>215</v>
@@ -11319,7 +11310,7 @@
         <v>30</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="F16" s="8">
         <v>0</v>
@@ -11327,7 +11318,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>217</v>
@@ -11339,7 +11330,7 @@
         <v>30</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="F17" s="8">
         <v>0</v>
@@ -11347,7 +11338,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>219</v>
@@ -11367,7 +11358,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>384</v>
@@ -11387,7 +11378,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>222</v>
@@ -11407,7 +11398,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>223</v>
@@ -11427,7 +11418,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>32</v>
@@ -11447,7 +11438,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>225</v>
@@ -11467,7 +11458,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>227</v>
@@ -11487,7 +11478,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>229</v>
@@ -11507,7 +11498,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>231</v>
@@ -11604,7 +11595,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>23</v>
@@ -11652,13 +11643,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="15" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B2" s="15" t="s">
         <v>68</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="D2" s="15" t="s">
         <v>23</v>
@@ -11669,13 +11660,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="15" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>68</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="D3" s="15" t="s">
         <v>23</v>
@@ -11684,13 +11675,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="15" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>68</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>23</v>
@@ -11699,13 +11690,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="15" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>68</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>23</v>
@@ -11714,13 +11705,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="15" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>68</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>23</v>
@@ -11735,7 +11726,7 @@
         <v>21</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>23</v>
@@ -11744,13 +11735,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="6" t="s">
+        <v>798</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>799</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>800</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>23</v>
@@ -11759,13 +11750,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="6" t="s">
+        <v>800</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="44" t="s">
         <v>801</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="48" t="s">
-        <v>802</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>23</v>
@@ -11774,13 +11765,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="6" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>68</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="D10" s="15" t="s">
         <v>23</v>
@@ -11789,7 +11780,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="6" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>8</v>
@@ -11798,7 +11789,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="E11" s="8"/>
     </row>
@@ -11835,7 +11826,7 @@
       <c r="D1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="47" t="s">
+      <c r="E1" s="43" t="s">
         <v>5</v>
       </c>
     </row>
@@ -11867,7 +11858,7 @@
         <v>9</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="E3" s="16">
         <v>0</v>
@@ -12518,274 +12509,274 @@
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="39" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="40" t="s">
+      <c r="A1" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="41" t="s">
+      <c r="F1" s="37" t="s">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B2" s="39" t="s">
         <v>763</v>
       </c>
-      <c r="B2" s="43" t="s">
+      <c r="C2" s="39" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="39" t="s">
         <v>764</v>
       </c>
-      <c r="C2" s="43" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="43" t="s">
+      <c r="F2" s="40">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B3" s="39" t="s">
+        <v>765</v>
+      </c>
+      <c r="C3" s="39" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="43" t="s">
-        <v>765</v>
-      </c>
-      <c r="F2" s="44">
-        <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="42" t="s">
-        <v>763</v>
-      </c>
-      <c r="B3" s="43" t="s">
+      <c r="E3" s="39" t="s">
         <v>766</v>
       </c>
-      <c r="C3" s="43" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="43" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="43" t="s">
+      <c r="F3" s="40">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B4" s="39" t="s">
         <v>767</v>
       </c>
-      <c r="F3" s="44">
-        <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="42" t="s">
-        <v>763</v>
-      </c>
-      <c r="B4" s="43" t="s">
+      <c r="C4" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="39" t="s">
         <v>768</v>
       </c>
-      <c r="C4" s="43" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="43" t="s">
+      <c r="E4" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="41"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B5" s="39" t="s">
         <v>769</v>
       </c>
-      <c r="E4" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="45"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="42" t="s">
-        <v>763</v>
-      </c>
-      <c r="B5" s="43" t="s">
+      <c r="C5" s="39" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="39" t="s">
         <v>770</v>
       </c>
-      <c r="C5" s="43" t="s">
+      <c r="E5" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="40">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B6" s="39" t="s">
+        <v>771</v>
+      </c>
+      <c r="C6" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="D5" s="43" t="s">
-        <v>771</v>
-      </c>
-      <c r="E5" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="44">
-        <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="42" t="s">
-        <v>763</v>
-      </c>
-      <c r="B6" s="43" t="s">
+      <c r="D6" s="39" t="s">
         <v>772</v>
       </c>
-      <c r="C6" s="43" t="s">
+      <c r="E6" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="40">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B7" s="39" t="s">
+        <v>773</v>
+      </c>
+      <c r="C7" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="39" t="s">
+        <v>774</v>
+      </c>
+      <c r="E7" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="41"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B8" s="39" t="s">
+        <v>775</v>
+      </c>
+      <c r="C8" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>776</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="41"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B9" s="39" t="s">
+        <v>777</v>
+      </c>
+      <c r="C9" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="D6" s="43" t="s">
-        <v>773</v>
-      </c>
-      <c r="E6" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="44">
-        <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="42" t="s">
-        <v>763</v>
-      </c>
-      <c r="B7" s="43" t="s">
-        <v>774</v>
-      </c>
-      <c r="C7" s="43" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="43" t="s">
-        <v>775</v>
-      </c>
-      <c r="E7" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="45"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="42" t="s">
-        <v>763</v>
-      </c>
-      <c r="B8" s="43" t="s">
-        <v>776</v>
-      </c>
-      <c r="C8" s="43" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="43" t="s">
-        <v>777</v>
-      </c>
-      <c r="E8" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="45"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="42" t="s">
-        <v>763</v>
-      </c>
-      <c r="B9" s="43" t="s">
+      <c r="D9" s="39" t="s">
         <v>778</v>
       </c>
-      <c r="C9" s="43" t="s">
+      <c r="E9" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="40">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B10" s="39" t="s">
+        <v>779</v>
+      </c>
+      <c r="C10" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="D9" s="43" t="s">
-        <v>779</v>
-      </c>
-      <c r="E9" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" s="44">
-        <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="42" t="s">
-        <v>763</v>
-      </c>
-      <c r="B10" s="43" t="s">
+      <c r="D10" s="39" t="s">
         <v>780</v>
       </c>
-      <c r="C10" s="43" t="s">
+      <c r="E10" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="40">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B11" s="39" t="s">
+        <v>489</v>
+      </c>
+      <c r="C11" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="39" t="s">
+        <v>781</v>
+      </c>
+      <c r="E11" s="39" t="s">
+        <v>490</v>
+      </c>
+      <c r="F11" s="40">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B12" s="39" t="s">
+        <v>491</v>
+      </c>
+      <c r="C12" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="39" t="s">
+        <v>781</v>
+      </c>
+      <c r="E12" s="39" t="s">
+        <v>492</v>
+      </c>
+      <c r="F12" s="40">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B13" s="39" t="s">
+        <v>782</v>
+      </c>
+      <c r="C13" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="39" t="s">
+        <v>783</v>
+      </c>
+      <c r="E13" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" s="41"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="A14" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="B14" s="38" t="s">
+        <v>784</v>
+      </c>
+      <c r="C14" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="43" t="s">
-        <v>781</v>
-      </c>
-      <c r="E10" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="44">
-        <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="42" t="s">
-        <v>763</v>
-      </c>
-      <c r="B11" s="43" t="s">
-        <v>489</v>
-      </c>
-      <c r="C11" s="43" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="43" t="s">
-        <v>782</v>
-      </c>
-      <c r="E11" s="43" t="s">
-        <v>490</v>
-      </c>
-      <c r="F11" s="44">
-        <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="42" t="s">
-        <v>763</v>
-      </c>
-      <c r="B12" s="43" t="s">
-        <v>491</v>
-      </c>
-      <c r="C12" s="43" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="43" t="s">
-        <v>782</v>
-      </c>
-      <c r="E12" s="43" t="s">
-        <v>492</v>
-      </c>
-      <c r="F12" s="44">
-        <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="42" t="s">
-        <v>763</v>
-      </c>
-      <c r="B13" s="43" t="s">
-        <v>783</v>
-      </c>
-      <c r="C13" s="43" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="43" t="s">
-        <v>784</v>
-      </c>
-      <c r="E13" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" s="45"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="42" t="s">
-        <v>763</v>
-      </c>
-      <c r="B14" s="42" t="s">
+      <c r="D14" s="38" t="s">
         <v>785</v>
       </c>
-      <c r="C14" s="42" t="s">
-        <v>68</v>
-      </c>
-      <c r="D14" s="42" t="s">
-        <v>786</v>
-      </c>
-      <c r="E14" s="42" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="46">
+      <c r="E14" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="42">
         <v>0</v>
       </c>
     </row>
@@ -12832,19 +12823,19 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="18" t="s">
+        <v>658</v>
+      </c>
+      <c r="B2" s="18" t="s">
         <v>659</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="C2" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="18" t="s">
         <v>660</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>661</v>
       </c>
       <c r="F2" s="19">
         <v>0</v>
@@ -12852,7 +12843,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B3" s="18" t="s">
         <v>7</v>
@@ -12860,7 +12851,7 @@
       <c r="C3" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="38" t="s">
+      <c r="D3" s="34" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="18" t="s">
@@ -12870,7 +12861,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>273</v>
@@ -12878,7 +12869,7 @@
       <c r="C4" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="34" t="s">
         <v>274</v>
       </c>
       <c r="E4" s="18" t="s">
@@ -12888,7 +12879,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>275</v>
@@ -12896,7 +12887,7 @@
       <c r="C5" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="D5" s="34" t="s">
         <v>77</v>
       </c>
       <c r="E5" s="18" t="s">
@@ -12908,7 +12899,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B6" s="18" t="s">
         <v>105</v>
@@ -12916,7 +12907,7 @@
       <c r="C6" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="38" t="s">
+      <c r="D6" s="34" t="s">
         <v>106</v>
       </c>
       <c r="E6" s="18" t="s">
@@ -12926,7 +12917,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B7" s="18" t="s">
         <v>13</v>
@@ -12934,7 +12925,7 @@
       <c r="C7" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="38" t="s">
+      <c r="D7" s="34" t="s">
         <v>171</v>
       </c>
       <c r="E7" s="18" t="s">
@@ -12944,7 +12935,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B8" s="18" t="s">
         <v>172</v>
@@ -12952,7 +12943,7 @@
       <c r="C8" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="38" t="s">
+      <c r="D8" s="34" t="s">
         <v>14</v>
       </c>
       <c r="E8" s="18" t="s">
@@ -12964,15 +12955,15 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="38" t="s">
+      <c r="D9" s="34" t="s">
         <v>14</v>
       </c>
       <c r="E9" s="18" t="s">
@@ -12984,7 +12975,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B10" s="18" t="s">
         <v>174</v>
@@ -12992,7 +12983,7 @@
       <c r="C10" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="38" t="s">
+      <c r="D10" s="34" t="s">
         <v>14</v>
       </c>
       <c r="E10" s="18" t="s">
@@ -13002,7 +12993,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B11" s="18" t="s">
         <v>176</v>
@@ -13010,7 +13001,7 @@
       <c r="C11" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="34" t="s">
         <v>14</v>
       </c>
       <c r="E11" s="18" t="s">
@@ -13022,16 +13013,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="C12" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="38" t="s">
-        <v>664</v>
+      <c r="D12" s="34" t="s">
+        <v>663</v>
       </c>
       <c r="E12" s="18" t="s">
         <v>23</v>
@@ -13040,16 +13031,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="C13" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="38" t="s">
-        <v>666</v>
+      <c r="D13" s="34" t="s">
+        <v>665</v>
       </c>
       <c r="E13" s="18" t="s">
         <v>23</v>
@@ -13060,16 +13051,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B14" s="18" t="s">
+        <v>666</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="34" t="s">
         <v>667</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="38" t="s">
-        <v>668</v>
       </c>
       <c r="E14" s="18" t="s">
         <v>23</v>
@@ -13080,16 +13071,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="C15" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D15" s="38" t="s">
-        <v>670</v>
+      <c r="D15" s="34" t="s">
+        <v>669</v>
       </c>
       <c r="E15" s="18" t="s">
         <v>23</v>
@@ -13098,16 +13089,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="C16" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D16" s="38" t="s">
-        <v>672</v>
+      <c r="D16" s="34" t="s">
+        <v>671</v>
       </c>
       <c r="E16" s="18" t="s">
         <v>23</v>
@@ -13116,16 +13107,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="C17" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D17" s="38" t="s">
-        <v>670</v>
+      <c r="D17" s="34" t="s">
+        <v>669</v>
       </c>
       <c r="E17" s="18" t="s">
         <v>23</v>
@@ -13134,16 +13125,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="C18" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="38" t="s">
-        <v>672</v>
+      <c r="D18" s="34" t="s">
+        <v>671</v>
       </c>
       <c r="E18" s="18" t="s">
         <v>23</v>
@@ -13154,16 +13145,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="C19" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D19" s="38" t="s">
-        <v>676</v>
+      <c r="D19" s="34" t="s">
+        <v>675</v>
       </c>
       <c r="E19" s="18" t="s">
         <v>23</v>
@@ -13172,32 +13163,32 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="C20" s="18" t="s">
         <v>68</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="E20" s="26"/>
       <c r="F20" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="C21" s="18" t="s">
         <v>68</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="E21" s="26"/>
       <c r="F21" s="7">
@@ -13206,19 +13197,19 @@
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B22" s="18" t="s">
+        <v>680</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="E22" s="18" t="s">
         <v>681</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>682</v>
       </c>
       <c r="F22" s="19">
         <v>0</v>
@@ -13226,34 +13217,34 @@
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B23" s="18" t="s">
+        <v>682</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="E23" s="18" t="s">
         <v>683</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>684</v>
       </c>
       <c r="F23" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="C24" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D24" s="38" t="s">
-        <v>686</v>
+      <c r="D24" s="34" t="s">
+        <v>685</v>
       </c>
       <c r="E24" s="18" t="s">
         <v>23</v>
@@ -13262,10 +13253,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="C25" s="18" t="s">
         <v>68</v>
@@ -13282,15 +13273,15 @@
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="C26" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D26" s="38" t="s">
+      <c r="D26" s="34" t="s">
         <v>381</v>
       </c>
       <c r="E26" s="18" t="s">
@@ -13300,7 +13291,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B27" s="18" t="s">
         <v>167</v>
@@ -13308,7 +13299,7 @@
       <c r="C27" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D27" s="38" t="s">
+      <c r="D27" s="34" t="s">
         <v>382</v>
       </c>
       <c r="E27" s="18" t="s">
@@ -13318,16 +13309,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="C28" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="38" t="s">
-        <v>690</v>
+      <c r="D28" s="34" t="s">
+        <v>689</v>
       </c>
       <c r="E28" s="18" t="s">
         <v>23</v>
@@ -13336,16 +13327,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
       <c r="A29" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="C29" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D29" s="38" t="s">
-        <v>692</v>
+      <c r="D29" s="34" t="s">
+        <v>691</v>
       </c>
       <c r="E29" s="18" t="s">
         <v>23</v>
@@ -13354,7 +13345,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B30" s="18" t="s">
         <v>384</v>
@@ -13362,7 +13353,7 @@
       <c r="C30" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D30" s="38" t="s">
+      <c r="D30" s="34" t="s">
         <v>385</v>
       </c>
       <c r="E30" s="18" t="s">
@@ -13372,15 +13363,15 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="C31" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D31" s="38" t="s">
+      <c r="D31" s="34" t="s">
         <v>14</v>
       </c>
       <c r="E31" s="18" t="s">
@@ -13390,19 +13381,19 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B32" s="18" t="s">
+        <v>693</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="E32" s="18" t="s">
         <v>694</v>
-      </c>
-      <c r="C32" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D32" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="E32" s="18" t="s">
-        <v>695</v>
       </c>
       <c r="F32" s="17">
         <v>1</v>
@@ -13410,33 +13401,33 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B33" s="18" t="s">
+        <v>695</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="E33" s="18" t="s">
         <v>696</v>
-      </c>
-      <c r="C33" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D33" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="E33" s="18" t="s">
-        <v>697</v>
       </c>
       <c r="F33" s="17"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C34" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="38" t="s">
+      <c r="D34" s="34" t="s">
         <v>77</v>
       </c>
       <c r="E34" s="18" t="s">
@@ -13448,16 +13439,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B35" s="18" t="s">
+        <v>698</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D35" s="34" t="s">
         <v>699</v>
-      </c>
-      <c r="C35" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D35" s="38" t="s">
-        <v>700</v>
       </c>
       <c r="E35" s="18" t="s">
         <v>23</v>
@@ -13466,16 +13457,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B36" s="18" t="s">
+        <v>700</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D36" s="34" t="s">
         <v>701</v>
-      </c>
-      <c r="C36" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D36" s="38" t="s">
-        <v>702</v>
       </c>
       <c r="E36" s="18" t="s">
         <v>23</v>
@@ -13484,16 +13475,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
       <c r="A37" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C37" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D37" s="38" t="s">
-        <v>704</v>
+      <c r="D37" s="34" t="s">
+        <v>703</v>
       </c>
       <c r="E37" s="18" t="s">
         <v>23</v>
@@ -13502,16 +13493,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
       <c r="A38" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C38" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D38" s="38" t="s">
-        <v>706</v>
+      <c r="D38" s="34" t="s">
+        <v>705</v>
       </c>
       <c r="E38" s="18" t="s">
         <v>23</v>
@@ -13520,16 +13511,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
       <c r="A39" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="C39" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D39" s="38" t="s">
-        <v>708</v>
+      <c r="D39" s="34" t="s">
+        <v>707</v>
       </c>
       <c r="E39" s="18" t="s">
         <v>23</v>
@@ -13538,7 +13529,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
       <c r="A40" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B40" s="18" t="s">
         <v>186</v>
@@ -13546,7 +13537,7 @@
       <c r="C40" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D40" s="38" t="s">
+      <c r="D40" s="34" t="s">
         <v>187</v>
       </c>
       <c r="E40" s="18" t="s">
@@ -13556,16 +13547,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
       <c r="A41" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="C41" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D41" s="38" t="s">
-        <v>710</v>
+      <c r="D41" s="34" t="s">
+        <v>709</v>
       </c>
       <c r="E41" s="18" t="s">
         <v>23</v>
@@ -13574,16 +13565,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
       <c r="A42" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="C42" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D42" s="38" t="s">
-        <v>712</v>
+      <c r="D42" s="34" t="s">
+        <v>711</v>
       </c>
       <c r="E42" s="18" t="s">
         <v>23</v>
@@ -13592,16 +13583,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
       <c r="A43" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B43" s="18" t="s">
+        <v>712</v>
+      </c>
+      <c r="C43" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D43" s="34" t="s">
         <v>713</v>
-      </c>
-      <c r="C43" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D43" s="38" t="s">
-        <v>714</v>
       </c>
       <c r="E43" s="18" t="s">
         <v>23</v>
@@ -13610,16 +13601,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
       <c r="A44" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="C44" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D44" s="38" t="s">
-        <v>716</v>
+      <c r="D44" s="34" t="s">
+        <v>715</v>
       </c>
       <c r="E44" s="18" t="s">
         <v>23</v>
@@ -13628,16 +13619,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
       <c r="A45" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B45" s="18" t="s">
+        <v>716</v>
+      </c>
+      <c r="C45" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D45" s="34" t="s">
         <v>717</v>
-      </c>
-      <c r="C45" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D45" s="38" t="s">
-        <v>718</v>
       </c>
       <c r="E45" s="18" t="s">
         <v>23</v>
@@ -13646,16 +13637,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
       <c r="A46" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B46" s="18" t="s">
+        <v>718</v>
+      </c>
+      <c r="C46" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D46" s="34" t="s">
         <v>719</v>
-      </c>
-      <c r="C46" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D46" s="38" t="s">
-        <v>720</v>
       </c>
       <c r="E46" s="18" t="s">
         <v>23</v>
@@ -13664,16 +13655,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
       <c r="A47" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B47" s="18" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="C47" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D47" s="38" t="s">
-        <v>722</v>
+      <c r="D47" s="34" t="s">
+        <v>721</v>
       </c>
       <c r="E47" s="18" t="s">
         <v>23</v>
@@ -13682,7 +13673,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
       <c r="A48" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B48" s="18" t="s">
         <v>654</v>
@@ -13690,7 +13681,7 @@
       <c r="C48" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D48" s="38" t="s">
+      <c r="D48" s="34" t="s">
         <v>655</v>
       </c>
       <c r="E48" s="18" t="s">
@@ -13700,15 +13691,15 @@
     </row>
     <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
       <c r="A49" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B49" s="18" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="C49" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D49" s="38" t="s">
+      <c r="D49" s="34" t="s">
         <v>77</v>
       </c>
       <c r="E49" s="18" t="s">
@@ -13720,16 +13711,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
       <c r="A50" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B50" s="18" t="s">
+        <v>723</v>
+      </c>
+      <c r="C50" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D50" s="34" t="s">
         <v>724</v>
-      </c>
-      <c r="C50" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D50" s="38" t="s">
-        <v>725</v>
       </c>
       <c r="E50" s="18" t="s">
         <v>23</v>
@@ -13738,16 +13729,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
       <c r="A51" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B51" s="18" t="s">
+        <v>725</v>
+      </c>
+      <c r="C51" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D51" s="34" t="s">
         <v>726</v>
-      </c>
-      <c r="C51" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D51" s="38" t="s">
-        <v>727</v>
       </c>
       <c r="E51" s="18" t="s">
         <v>23</v>
@@ -13758,16 +13749,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
       <c r="A52" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B52" s="18" t="s">
+        <v>727</v>
+      </c>
+      <c r="C52" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D52" s="34" t="s">
         <v>728</v>
-      </c>
-      <c r="C52" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D52" s="38" t="s">
-        <v>729</v>
       </c>
       <c r="E52" s="18" t="s">
         <v>23</v>
@@ -13778,16 +13769,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
       <c r="A53" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B53" s="18" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="C53" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D53" s="38" t="s">
-        <v>731</v>
+      <c r="D53" s="34" t="s">
+        <v>730</v>
       </c>
       <c r="E53" s="18" t="s">
         <v>164</v>
@@ -13796,34 +13787,34 @@
     </row>
     <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
       <c r="A54" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B54" s="18" t="s">
+        <v>731</v>
+      </c>
+      <c r="C54" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D54" s="34" t="s">
         <v>732</v>
       </c>
-      <c r="C54" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D54" s="38" t="s">
-        <v>733</v>
-      </c>
       <c r="E54" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F54" s="38"/>
+      <c r="F54" s="34"/>
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
       <c r="A55" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="C55" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D55" s="38" t="s">
-        <v>735</v>
+      <c r="D55" s="34" t="s">
+        <v>734</v>
       </c>
       <c r="E55" s="18" t="s">
         <v>23</v>
@@ -13832,16 +13823,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
       <c r="A56" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B56" s="18" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C56" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D56" s="38" t="s">
-        <v>737</v>
+      <c r="D56" s="34" t="s">
+        <v>736</v>
       </c>
       <c r="E56" s="18" t="s">
         <v>23</v>
@@ -13850,16 +13841,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
       <c r="A57" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B57" s="18" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="C57" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D57" s="38" t="s">
-        <v>739</v>
+      <c r="D57" s="34" t="s">
+        <v>738</v>
       </c>
       <c r="E57" s="18" t="s">
         <v>23</v>
@@ -13868,16 +13859,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
       <c r="A58" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B58" s="18" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="C58" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D58" s="38" t="s">
-        <v>737</v>
+      <c r="D58" s="34" t="s">
+        <v>736</v>
       </c>
       <c r="E58" s="18" t="s">
         <v>23</v>
@@ -13886,16 +13877,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
       <c r="A59" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B59" s="18" t="s">
+        <v>740</v>
+      </c>
+      <c r="C59" s="18" t="s">
         <v>741</v>
       </c>
-      <c r="C59" s="18" t="s">
+      <c r="D59" s="34" t="s">
         <v>742</v>
-      </c>
-      <c r="D59" s="38" t="s">
-        <v>743</v>
       </c>
       <c r="E59" s="18" t="s">
         <v>23</v>
@@ -13904,16 +13895,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
       <c r="A60" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B60" s="18" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="C60" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D60" s="38" t="s">
-        <v>745</v>
+      <c r="D60" s="34" t="s">
+        <v>744</v>
       </c>
       <c r="E60" s="18" t="s">
         <v>23</v>
@@ -13922,16 +13913,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
       <c r="A61" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B61" s="18" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="C61" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D61" s="38" t="s">
-        <v>745</v>
+      <c r="D61" s="34" t="s">
+        <v>744</v>
       </c>
       <c r="E61" s="18" t="s">
         <v>23</v>
@@ -13942,16 +13933,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
       <c r="A62" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B62" s="18" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="C62" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D62" s="38" t="s">
-        <v>737</v>
+      <c r="D62" s="34" t="s">
+        <v>736</v>
       </c>
       <c r="E62" s="18" t="s">
         <v>23</v>
@@ -13960,16 +13951,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
       <c r="A63" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B63" s="18" t="s">
+        <v>747</v>
+      </c>
+      <c r="C63" s="18" t="s">
+        <v>741</v>
+      </c>
+      <c r="D63" s="34" t="s">
         <v>748</v>
-      </c>
-      <c r="C63" s="18" t="s">
-        <v>742</v>
-      </c>
-      <c r="D63" s="38" t="s">
-        <v>749</v>
       </c>
       <c r="E63" s="18" t="s">
         <v>23</v>
@@ -13978,19 +13969,19 @@
     </row>
     <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="19.5">
       <c r="A64" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B64" s="18" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="C64" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D64" s="38" t="s">
+      <c r="D64" s="34" t="s">
         <v>14</v>
       </c>
       <c r="E64" s="18" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F64" s="19">
         <v>1</v>
@@ -13998,16 +13989,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="19.5">
       <c r="A65" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B65" s="18" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="C65" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D65" s="38" t="s">
-        <v>752</v>
+      <c r="D65" s="34" t="s">
+        <v>751</v>
       </c>
       <c r="E65" s="18" t="s">
         <v>23</v>
@@ -14016,16 +14007,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
       <c r="A66" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B66" s="18" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="C66" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D66" s="38" t="s">
-        <v>754</v>
+      <c r="D66" s="34" t="s">
+        <v>753</v>
       </c>
       <c r="E66" s="18" t="s">
         <v>23</v>
@@ -14034,16 +14025,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
       <c r="A67" s="26" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B67" s="26" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="C67" s="26" t="s">
         <v>25</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="E67" s="26" t="s">
         <v>23</v>
@@ -14052,16 +14043,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
       <c r="A68" s="26" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B68" s="26" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="C68" s="26" t="s">
         <v>25</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="E68" s="26" t="s">
         <v>23</v>
@@ -14070,16 +14061,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
       <c r="A69" s="26" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B69" s="26" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="C69" s="26" t="s">
         <v>25</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="E69" s="26" t="s">
         <v>23</v>
@@ -14088,16 +14079,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="19.5">
       <c r="A70" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B70" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="C70" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D70" s="34" t="s">
         <v>761</v>
-      </c>
-      <c r="C70" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D70" s="38" t="s">
-        <v>762</v>
       </c>
       <c r="E70" s="18" t="s">
         <v>23</v>
@@ -14125,7 +14116,7 @@
     <col min="6" max="6" style="11" width="23.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -14145,7 +14136,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="6" t="s">
         <v>599</v>
       </c>
@@ -14165,7 +14156,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="6" t="s">
         <v>599</v>
       </c>
@@ -14185,7 +14176,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="6" t="s">
         <v>599</v>
       </c>
@@ -14205,7 +14196,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="6" t="s">
         <v>599</v>
       </c>
@@ -14225,7 +14216,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="6" t="s">
         <v>599</v>
       </c>
@@ -14245,7 +14236,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="6" t="s">
         <v>599</v>
       </c>
@@ -14265,7 +14256,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="6" t="s">
         <v>599</v>
       </c>
@@ -14285,7 +14276,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="6" t="s">
         <v>599</v>
       </c>
@@ -14305,7 +14296,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="6" t="s">
         <v>599</v>
       </c>
@@ -14325,7 +14316,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="6" t="s">
         <v>599</v>
       </c>
@@ -14345,7 +14336,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="6" t="s">
         <v>599</v>
       </c>
@@ -14365,7 +14356,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="6" t="s">
         <v>599</v>
       </c>
@@ -14385,7 +14376,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="6" t="s">
         <v>599</v>
       </c>
@@ -14405,7 +14396,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="6" t="s">
         <v>599</v>
       </c>
@@ -14425,7 +14416,7 @@
         <v>598</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="6" t="s">
         <v>599</v>
       </c>
@@ -14814,44 +14805,20 @@
       <c r="F35" s="33"/>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
-      <c r="A36" s="34" t="s">
-        <v>658</v>
-      </c>
-      <c r="B36" s="35" t="s">
-        <v>658</v>
-      </c>
-      <c r="C36" s="35" t="s">
-        <v>658</v>
-      </c>
-      <c r="D36" s="35" t="s">
-        <v>658</v>
-      </c>
-      <c r="E36" s="35" t="s">
-        <v>658</v>
-      </c>
-      <c r="F36" s="36" t="s">
-        <v>658</v>
-      </c>
+      <c r="A36" s="6"/>
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="17"/>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
-      <c r="A37" s="34" t="s">
-        <v>658</v>
-      </c>
-      <c r="B37" s="34" t="s">
-        <v>658</v>
-      </c>
-      <c r="C37" s="34" t="s">
-        <v>658</v>
-      </c>
-      <c r="D37" s="34" t="s">
-        <v>658</v>
-      </c>
-      <c r="E37" s="34" t="s">
-        <v>658</v>
-      </c>
-      <c r="F37" s="37" t="s">
-        <v>658</v>
-      </c>
+      <c r="A37" s="6"/>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>